<commit_message>
fix: copy nginx.prod.conf to container and fix port mapping
</commit_message>
<xml_diff>
--- a/demodata/ZRFI005.XLSX
+++ b/demodata/ZRFI005.XLSX
@@ -15,14 +15,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Y$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Y$100</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="985" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="273">
   <si>
     <t>1000</t>
   </si>
@@ -330,403 +330,418 @@
     <t>CÔNG TY TNHH MILLENNIUM FURNITURE</t>
   </si>
   <si>
+    <t>10810655</t>
+  </si>
+  <si>
+    <t>PHẠM BÍCH THỦY</t>
+  </si>
+  <si>
+    <t>1200000834</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH TM DV XD TĂNG PHI</t>
+  </si>
+  <si>
+    <t>31</t>
+  </si>
+  <si>
+    <t>10810746</t>
+  </si>
+  <si>
+    <t>LÊ VĂN TẤN</t>
+  </si>
+  <si>
+    <t>1200000839</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH HỒNG ÂN</t>
+  </si>
+  <si>
+    <t>10811384</t>
+  </si>
+  <si>
+    <t>VÕ THANH TUẤN</t>
+  </si>
+  <si>
+    <t>1200000842</t>
+  </si>
+  <si>
+    <t>DOANH NGHIỆP TƯ NHÂN THANH SƯƠNG</t>
+  </si>
+  <si>
+    <t>1200000843</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH MỘT THÀNH VIÊN CÔNG HẬU</t>
+  </si>
+  <si>
+    <t>1200000849</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH XÂY DỰNG THƯƠNG MẠI HOÀNG NGỌC THANH</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>1200000850</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SƠN KIM PHÚC PU</t>
+  </si>
+  <si>
+    <t>1200000851</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI DỊCH VỤ PHẠM GIA TUẤN</t>
+  </si>
+  <si>
+    <t>1200000852</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI - XÂY DỰNG THIÊN HÀ PHÁT</t>
+  </si>
+  <si>
+    <t>10110766</t>
+  </si>
+  <si>
+    <t>PHẠM MINH SĨ</t>
+  </si>
+  <si>
+    <t>1200000854</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH TRẦN LIÊN HƯNG</t>
+  </si>
+  <si>
+    <t>1200000856</t>
+  </si>
+  <si>
+    <t>CÔNG TY TRÁCH NHIỆM HỮU HẠN AN PHÚ</t>
+  </si>
+  <si>
+    <t>1200000857</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ DANH PHÁT</t>
+  </si>
+  <si>
+    <t>1200000859</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH MỘT THÀNH VIÊN SẢN XUẤT THƯƠNG MẠI LOUIS PHƯỚC THẠNH</t>
+  </si>
+  <si>
+    <t>1200000864</t>
+  </si>
+  <si>
+    <t>CHÂU HOÀNG ANH THY (HỘ KINH DOANH VĨNH LỘC)</t>
+  </si>
+  <si>
+    <t>1200000865</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH VẬT LIỆU XÂY DỰNG NGỌC THANH MINH</t>
+  </si>
+  <si>
+    <t>62</t>
+  </si>
+  <si>
+    <t>1200000867</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH KINH DOANH NAM PHÁT</t>
+  </si>
+  <si>
+    <t>1200000882</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI DỊCH VỤ XÂY DỰNG VÀ CÔNG NGHỆ SÀN SƠN PHÁT</t>
+  </si>
+  <si>
+    <t>1200000888</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH ZOE FURNITURE</t>
+  </si>
+  <si>
+    <t>1200000903</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH CÔNG NGHIỆP NHÀ XANH</t>
+  </si>
+  <si>
+    <t>10811780</t>
+  </si>
+  <si>
+    <t>TẠ DUY HÀ</t>
+  </si>
+  <si>
+    <t>1200000904</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH BẢO LÂM</t>
+  </si>
+  <si>
+    <t>1200000935</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN HỆ THỐNG SIÊU THỊ SƠN</t>
+  </si>
+  <si>
+    <t>1200000949</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN BAO BÌ IN KIM LOẠI THẾ KỶ</t>
+  </si>
+  <si>
+    <t>1200000963</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH CƠ KHÍ XÂY DỰNG VIỆT THẮNG</t>
+  </si>
+  <si>
+    <t>1200000971</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ SƠN ANH TÚ</t>
+  </si>
+  <si>
+    <t>1200000973</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH AN THỊNH FURNITURE</t>
+  </si>
+  <si>
+    <t>1200000992</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH DV KT AN TÂM PHÁT</t>
+  </si>
+  <si>
+    <t>1200001011</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN ĐÔNG NGÔ MANUFACTURER</t>
+  </si>
+  <si>
+    <t>1200001023</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI - DỊCH VỤ - XÂY DỰNG MAI TÂM</t>
+  </si>
+  <si>
+    <t>1200001029</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH TRANG TRÍ NỘI THẤT PHONG THẢO</t>
+  </si>
+  <si>
+    <t>10400773</t>
+  </si>
+  <si>
+    <t>VŨ ANH HAI</t>
+  </si>
+  <si>
+    <t>1200001038</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH PHÚ MỸ THĂNG</t>
+  </si>
+  <si>
+    <t>1200001041</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI XÂY DỰNG THIÊN PHÚ DECOR</t>
+  </si>
+  <si>
+    <t>1200001042</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH KIẾN TRÚC GỖ BỌC ĐÔ</t>
+  </si>
+  <si>
+    <t>1200001051</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH VINAWOOD</t>
+  </si>
+  <si>
+    <t>10999776</t>
+  </si>
+  <si>
+    <t>ĐẶNG VĂN CHỈ</t>
+  </si>
+  <si>
+    <t>1200001056</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI THANH THANH LIÊM</t>
+  </si>
+  <si>
+    <t>1200001062</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN BOHO CORPORATION</t>
+  </si>
+  <si>
+    <t>1200001065</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ TÂN LÂM</t>
+  </si>
+  <si>
+    <t>1200001072</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH MỘT THÀNH VIÊN KIM CHI</t>
+  </si>
+  <si>
+    <t>1200001077</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SX TM QUANG TRUNG NGUYÊN</t>
+  </si>
+  <si>
+    <t>1200001079</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI - XÂY DỰNG HUY HƯNG</t>
+  </si>
+  <si>
+    <t>1200001084</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SX TM DV SƠN MIỀN TÂY</t>
+  </si>
+  <si>
+    <t>1200001087</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SX-TM SÀI GÒN RIVER VIỆT NAM</t>
+  </si>
+  <si>
+    <t>1200001092</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH HỒNG LUÂN 3</t>
+  </si>
+  <si>
+    <t>1200001094</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH TM SẢN XUẤT XNK NỘI THẤT MCS</t>
+  </si>
+  <si>
+    <t>1200001104</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN ARTEX ĐỒNG THÁP</t>
+  </si>
+  <si>
+    <t>1200001109</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI DỊCH VỤ XÂY DỰNG THIÊN ĐỊNH</t>
+  </si>
+  <si>
+    <t>1200001113</t>
+  </si>
+  <si>
+    <t>CÔNG TY TRÁCH NHIỆM HỮU HẠN XD SX TM DV AB</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>1200001114</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI TUÝP NHÔM THUẬN QUÂN</t>
+  </si>
+  <si>
+    <t>1200001118</t>
+  </si>
+  <si>
+    <t>LAZADA</t>
+  </si>
+  <si>
+    <t>1200001119</t>
+  </si>
+  <si>
+    <t>VŨ ĐÌNH DŨNG</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>1200001120</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH TRANSFORMER ROBOTICS PTE</t>
+  </si>
+  <si>
+    <t>1200001123</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SƠN TÀI TRÍ</t>
+  </si>
+  <si>
+    <t>1200001124</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH MTV HOÀNG MINH TUẤN</t>
+  </si>
+  <si>
+    <t>1200001125</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH TRẦN QUÝ</t>
+  </si>
+  <si>
+    <t>1200001144</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH BUÔN LÊ COFFEE</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>1300000002</t>
+  </si>
+  <si>
+    <t>KODA WOODCRAFT SDN BHD</t>
+  </si>
+  <si>
+    <t>1200000863</t>
+  </si>
+  <si>
+    <t>Công Ty TNHH Thương Mại Tổng Hợp Dũng Lý</t>
+  </si>
+  <si>
+    <t>1200000974</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH CAO VÕ</t>
+  </si>
+  <si>
+    <t>1200001004</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH MỘT THÀNH VIÊN XÂY DỰNG - THƯƠNG MẠI VÀ DỊCH VỤ HOÀNG GIA</t>
+  </si>
+  <si>
     <t>1200000820</t>
   </si>
   <si>
     <t>CÔNG TY TNHH SẢN XUẤT NỘI THẤT TRẦN TIẾN</t>
   </si>
   <si>
-    <t>10810655</t>
-  </si>
-  <si>
-    <t>PHẠM BÍCH THỦY</t>
-  </si>
-  <si>
-    <t>1200000834</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH TM DV XD TĂNG PHI</t>
-  </si>
-  <si>
-    <t>31</t>
-  </si>
-  <si>
-    <t>10810746</t>
-  </si>
-  <si>
-    <t>LÊ VĂN TẤN</t>
-  </si>
-  <si>
-    <t>1200000839</t>
-  </si>
-  <si>
-    <t>HỘ KINH DOANH HỒNG ÂN</t>
-  </si>
-  <si>
-    <t>10811384</t>
-  </si>
-  <si>
-    <t>VÕ THANH TUẤN</t>
-  </si>
-  <si>
-    <t>1200000842</t>
-  </si>
-  <si>
-    <t>DOANH NGHIỆP TƯ NHÂN THANH SƯƠNG</t>
-  </si>
-  <si>
-    <t>1200000843</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH MỘT THÀNH VIÊN CÔNG HẬU</t>
-  </si>
-  <si>
-    <t>1200000849</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH XÂY DỰNG THƯƠNG MẠI HOÀNG NGỌC THANH</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>1200000850</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SƠN KIM PHÚC PU</t>
-  </si>
-  <si>
-    <t>1200000851</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI DỊCH VỤ PHẠM GIA TUẤN</t>
-  </si>
-  <si>
-    <t>1200000852</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI - XÂY DỰNG THIÊN HÀ PHÁT</t>
-  </si>
-  <si>
-    <t>10110766</t>
-  </si>
-  <si>
-    <t>PHẠM MINH SĨ</t>
-  </si>
-  <si>
-    <t>1200000854</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH TRẦN LIÊN HƯNG</t>
-  </si>
-  <si>
-    <t>1200000856</t>
-  </si>
-  <si>
-    <t>CÔNG TY TRÁCH NHIỆM HỮU HẠN AN PHÚ</t>
-  </si>
-  <si>
-    <t>1200000857</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ DANH PHÁT</t>
-  </si>
-  <si>
-    <t>1200000859</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH MỘT THÀNH VIÊN SẢN XUẤT THƯƠNG MẠI LOUIS PHƯỚC THẠNH</t>
-  </si>
-  <si>
-    <t>1200000864</t>
-  </si>
-  <si>
-    <t>CHÂU HOÀNG ANH THY (HỘ KINH DOANH VĨNH LỘC)</t>
-  </si>
-  <si>
-    <t>1200000865</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH VẬT LIỆU XÂY DỰNG NGỌC THANH MINH</t>
-  </si>
-  <si>
-    <t>62</t>
-  </si>
-  <si>
-    <t>1200000867</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH KINH DOANH NAM PHÁT</t>
-  </si>
-  <si>
-    <t>1200000882</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI DỊCH VỤ XÂY DỰNG VÀ CÔNG NGHỆ SÀN SƠN PHÁT</t>
-  </si>
-  <si>
-    <t>1200000903</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH CÔNG NGHIỆP NHÀ XANH</t>
-  </si>
-  <si>
-    <t>10811780</t>
-  </si>
-  <si>
-    <t>TẠ DUY HÀ</t>
-  </si>
-  <si>
-    <t>1200000904</t>
-  </si>
-  <si>
-    <t>HỘ KINH DOANH BẢO LÂM</t>
-  </si>
-  <si>
     <t>1200000922</t>
   </si>
   <si>
     <t>CÔNG TY TNHH THƯƠNG MẠI XÂY DỰNG TRANG TRÍ NỘI THẤT THỊNH HƯNG</t>
-  </si>
-  <si>
-    <t>1200000935</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN HỆ THỐNG SIÊU THỊ SƠN</t>
-  </si>
-  <si>
-    <t>1200000949</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN BAO BÌ IN KIM LOẠI THẾ KỶ</t>
-  </si>
-  <si>
-    <t>1200000963</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH CƠ KHÍ XÂY DỰNG VIỆT THẮNG</t>
-  </si>
-  <si>
-    <t>1200000971</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ SƠN ANH TÚ</t>
-  </si>
-  <si>
-    <t>1200000973</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH AN THỊNH FURNITURE</t>
-  </si>
-  <si>
-    <t>1200000992</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH DV KT AN TÂM PHÁT</t>
-  </si>
-  <si>
-    <t>1200001011</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN ĐÔNG NGÔ MANUFACTURER</t>
-  </si>
-  <si>
-    <t>1200001023</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI - DỊCH VỤ - XÂY DỰNG MAI TÂM</t>
-  </si>
-  <si>
-    <t>1200001029</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH TRANG TRÍ NỘI THẤT PHONG THẢO</t>
-  </si>
-  <si>
-    <t>10400773</t>
-  </si>
-  <si>
-    <t>VŨ ANH HAI</t>
-  </si>
-  <si>
-    <t>1200001038</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH PHÚ MỸ THĂNG</t>
-  </si>
-  <si>
-    <t>1200001041</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI XÂY DỰNG THIÊN PHÚ DECOR</t>
-  </si>
-  <si>
-    <t>1200001042</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH KIẾN TRÚC GỖ BỌC ĐÔ</t>
-  </si>
-  <si>
-    <t>1200001051</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH VINAWOOD</t>
-  </si>
-  <si>
-    <t>10999776</t>
-  </si>
-  <si>
-    <t>ĐẶNG VĂN CHỈ</t>
-  </si>
-  <si>
-    <t>1200001056</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI THANH THANH LIÊM</t>
-  </si>
-  <si>
-    <t>1200001062</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN BOHO CORPORATION</t>
-  </si>
-  <si>
-    <t>1200001065</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ TÂN LÂM</t>
-  </si>
-  <si>
-    <t>1200001072</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH MỘT THÀNH VIÊN KIM CHI</t>
-  </si>
-  <si>
-    <t>1200001077</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SX TM QUANG TRUNG NGUYÊN</t>
-  </si>
-  <si>
-    <t>1200001079</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI - XÂY DỰNG HUY HƯNG</t>
-  </si>
-  <si>
-    <t>1200001084</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SX TM DV SƠN MIỀN TÂY</t>
-  </si>
-  <si>
-    <t>1200001087</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SX-TM SÀI GÒN RIVER VIỆT NAM</t>
-  </si>
-  <si>
-    <t>1200001092</t>
-  </si>
-  <si>
-    <t>HỘ KINH DOANH HỒNG LUÂN 3</t>
-  </si>
-  <si>
-    <t>1200001094</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH TM SẢN XUẤT XNK NỘI THẤT MCS</t>
-  </si>
-  <si>
-    <t>1200001104</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN ARTEX ĐỒNG THÁP</t>
-  </si>
-  <si>
-    <t>1200001109</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI DỊCH VỤ XÂY DỰNG THIÊN ĐỊNH</t>
-  </si>
-  <si>
-    <t>1200001113</t>
-  </si>
-  <si>
-    <t>CÔNG TY TRÁCH NHIỆM HỮU HẠN XD SX TM DV AB</t>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>1200001114</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI TUÝP NHÔM THUẬN QUÂN</t>
-  </si>
-  <si>
-    <t>1200001118</t>
-  </si>
-  <si>
-    <t>LAZADA</t>
-  </si>
-  <si>
-    <t>1200001119</t>
-  </si>
-  <si>
-    <t>VŨ ĐÌNH DŨNG</t>
-  </si>
-  <si>
-    <t>1200001123</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SƠN TÀI TRÍ</t>
-  </si>
-  <si>
-    <t>1200001124</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH MTV HOÀNG MINH TUẤN</t>
-  </si>
-  <si>
-    <t>1200001125</t>
-  </si>
-  <si>
-    <t>HỘ KINH DOANH TRẦN QUÝ</t>
-  </si>
-  <si>
-    <t>1200001144</t>
-  </si>
-  <si>
-    <t>HỘ KINH DOANH BUÔN LÊ COFFEE</t>
-  </si>
-  <si>
-    <t>06</t>
-  </si>
-  <si>
-    <t>1300000002</t>
-  </si>
-  <si>
-    <t>KODA WOODCRAFT SDN BHD</t>
-  </si>
-  <si>
-    <t>1200000863</t>
-  </si>
-  <si>
-    <t>Công Ty TNHH Thương Mại Tổng Hợp Dũng Lý</t>
-  </si>
-  <si>
-    <t>1200000974</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH CAO VÕ</t>
-  </si>
-  <si>
-    <t>1200001004</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH MỘT THÀNH VIÊN XÂY DỰNG - THƯƠNG MẠI VÀ DỊCH VỤ HOÀNG GIA</t>
   </si>
   <si>
     <t>1200000769</t>
@@ -1172,7 +1187,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y97"/>
+  <dimension ref="A1:Y100"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -1201,79 +1216,79 @@
   <sheetData>
     <row r="1" spans="1:25" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
@@ -2028,7 +2043,7 @@
         <v>0</v>
       </c>
       <c r="T11" s="2">
-        <v>0</v>
+        <v>707423134</v>
       </c>
       <c r="U11" s="2">
         <v>0</v>
@@ -2043,7 +2058,7 @@
         <v>0</v>
       </c>
       <c r="Y11" s="2">
-        <v>0</v>
+        <v>707423134</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
@@ -3902,31 +3917,31 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D36" t="s">
         <v>3</v>
       </c>
       <c r="E36" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F36" t="s">
-        <v>5</v>
+        <v>102</v>
       </c>
       <c r="G36" t="s">
-        <v>6</v>
+        <v>103</v>
       </c>
       <c r="H36" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="I36" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="J36" t="s">
         <v>9</v>
       </c>
       <c r="K36" s="2">
-        <v>10069920</v>
+        <v>68591463</v>
       </c>
       <c r="L36" s="2">
         <v>0</v>
@@ -3944,7 +3959,7 @@
         <v>0</v>
       </c>
       <c r="Q36" s="2">
-        <v>10069920</v>
+        <v>68591463</v>
       </c>
       <c r="R36" s="2">
         <v>0</v>
@@ -3985,28 +4000,28 @@
         <v>3</v>
       </c>
       <c r="E37" t="s">
-        <v>80</v>
+        <v>106</v>
       </c>
       <c r="F37" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="G37" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="H37" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="I37" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="J37" t="s">
         <v>9</v>
       </c>
       <c r="K37" s="2">
-        <v>68591463</v>
+        <v>23259938</v>
       </c>
       <c r="L37" s="2">
-        <v>0</v>
+        <v>9321398</v>
       </c>
       <c r="M37" s="2">
         <v>0</v>
@@ -4021,7 +4036,7 @@
         <v>0</v>
       </c>
       <c r="Q37" s="2">
-        <v>68591463</v>
+        <v>32581336</v>
       </c>
       <c r="R37" s="2">
         <v>0</v>
@@ -4062,28 +4077,28 @@
         <v>3</v>
       </c>
       <c r="E38" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="F38" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="G38" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="H38" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="I38" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="J38" t="s">
         <v>9</v>
       </c>
       <c r="K38" s="2">
-        <v>23259938</v>
+        <v>68546328</v>
       </c>
       <c r="L38" s="2">
-        <v>9321398</v>
+        <v>0</v>
       </c>
       <c r="M38" s="2">
         <v>0</v>
@@ -4098,13 +4113,13 @@
         <v>0</v>
       </c>
       <c r="Q38" s="2">
-        <v>32581336</v>
+        <v>68546328</v>
       </c>
       <c r="R38" s="2">
         <v>0</v>
       </c>
       <c r="S38" s="2">
-        <v>0</v>
+        <v>23886291</v>
       </c>
       <c r="T38" s="2">
         <v>0</v>
@@ -4122,7 +4137,7 @@
         <v>0</v>
       </c>
       <c r="Y38" s="2">
-        <v>0</v>
+        <v>23886291</v>
       </c>
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.25">
@@ -4142,10 +4157,10 @@
         <v>80</v>
       </c>
       <c r="F39" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G39" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H39" t="s">
         <v>115</v>
@@ -4157,10 +4172,10 @@
         <v>9</v>
       </c>
       <c r="K39" s="2">
-        <v>68546328</v>
+        <v>587755726</v>
       </c>
       <c r="L39" s="2">
-        <v>0</v>
+        <v>424340449</v>
       </c>
       <c r="M39" s="2">
         <v>0</v>
@@ -4175,16 +4190,16 @@
         <v>0</v>
       </c>
       <c r="Q39" s="2">
-        <v>68546328</v>
+        <v>1012096175</v>
       </c>
       <c r="R39" s="2">
         <v>0</v>
       </c>
       <c r="S39" s="2">
-        <v>23886291</v>
+        <v>0</v>
       </c>
       <c r="T39" s="2">
-        <v>0</v>
+        <v>200000000</v>
       </c>
       <c r="U39" s="2">
         <v>0</v>
@@ -4199,7 +4214,7 @@
         <v>0</v>
       </c>
       <c r="Y39" s="2">
-        <v>23886291</v>
+        <v>200000000</v>
       </c>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.25">
@@ -4219,10 +4234,10 @@
         <v>80</v>
       </c>
       <c r="F40" t="s">
-        <v>113</v>
+        <v>102</v>
       </c>
       <c r="G40" t="s">
-        <v>114</v>
+        <v>103</v>
       </c>
       <c r="H40" t="s">
         <v>117</v>
@@ -4234,10 +4249,10 @@
         <v>9</v>
       </c>
       <c r="K40" s="2">
-        <v>587755726</v>
+        <v>305651559</v>
       </c>
       <c r="L40" s="2">
-        <v>424340449</v>
+        <v>0</v>
       </c>
       <c r="M40" s="2">
         <v>0</v>
@@ -4252,13 +4267,13 @@
         <v>0</v>
       </c>
       <c r="Q40" s="2">
-        <v>1012096175</v>
+        <v>305651559</v>
       </c>
       <c r="R40" s="2">
         <v>0</v>
       </c>
       <c r="S40" s="2">
-        <v>0</v>
+        <v>48581001</v>
       </c>
       <c r="T40" s="2">
         <v>0</v>
@@ -4276,7 +4291,7 @@
         <v>0</v>
       </c>
       <c r="Y40" s="2">
-        <v>0</v>
+        <v>48581001</v>
       </c>
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.25">
@@ -4293,25 +4308,25 @@
         <v>3</v>
       </c>
       <c r="E41" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="F41" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="G41" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="H41" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="I41" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="J41" t="s">
         <v>9</v>
       </c>
       <c r="K41" s="2">
-        <v>305651559</v>
+        <v>0</v>
       </c>
       <c r="L41" s="2">
         <v>0</v>
@@ -4320,7 +4335,7 @@
         <v>0</v>
       </c>
       <c r="N41" s="2">
-        <v>0</v>
+        <v>36336913</v>
       </c>
       <c r="O41" s="2">
         <v>0</v>
@@ -4329,13 +4344,13 @@
         <v>0</v>
       </c>
       <c r="Q41" s="2">
-        <v>305651559</v>
+        <v>36336913</v>
       </c>
       <c r="R41" s="2">
         <v>0</v>
       </c>
       <c r="S41" s="2">
-        <v>48581001</v>
+        <v>0</v>
       </c>
       <c r="T41" s="2">
         <v>0</v>
@@ -4353,7 +4368,7 @@
         <v>0</v>
       </c>
       <c r="Y41" s="2">
-        <v>48581001</v>
+        <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:25" x14ac:dyDescent="0.25">
@@ -4370,13 +4385,13 @@
         <v>3</v>
       </c>
       <c r="E42" t="s">
-        <v>121</v>
+        <v>80</v>
       </c>
       <c r="F42" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G42" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H42" t="s">
         <v>122</v>
@@ -4388,7 +4403,7 @@
         <v>9</v>
       </c>
       <c r="K42" s="2">
-        <v>0</v>
+        <v>430866875</v>
       </c>
       <c r="L42" s="2">
         <v>0</v>
@@ -4397,7 +4412,7 @@
         <v>0</v>
       </c>
       <c r="N42" s="2">
-        <v>36336913</v>
+        <v>0</v>
       </c>
       <c r="O42" s="2">
         <v>0</v>
@@ -4406,13 +4421,13 @@
         <v>0</v>
       </c>
       <c r="Q42" s="2">
-        <v>36336913</v>
+        <v>430866875</v>
       </c>
       <c r="R42" s="2">
         <v>0</v>
       </c>
       <c r="S42" s="2">
-        <v>0</v>
+        <v>144789230</v>
       </c>
       <c r="T42" s="2">
         <v>0</v>
@@ -4430,7 +4445,7 @@
         <v>0</v>
       </c>
       <c r="Y42" s="2">
-        <v>0</v>
+        <v>144789230</v>
       </c>
     </row>
     <row r="43" spans="1:25" x14ac:dyDescent="0.25">
@@ -4450,10 +4465,10 @@
         <v>80</v>
       </c>
       <c r="F43" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="G43" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="H43" t="s">
         <v>124</v>
@@ -4465,7 +4480,7 @@
         <v>9</v>
       </c>
       <c r="K43" s="2">
-        <v>430866875</v>
+        <v>316905738</v>
       </c>
       <c r="L43" s="2">
         <v>0</v>
@@ -4483,13 +4498,13 @@
         <v>0</v>
       </c>
       <c r="Q43" s="2">
-        <v>430866875</v>
+        <v>316905738</v>
       </c>
       <c r="R43" s="2">
         <v>0</v>
       </c>
       <c r="S43" s="2">
-        <v>144789230</v>
+        <v>0</v>
       </c>
       <c r="T43" s="2">
         <v>0</v>
@@ -4507,7 +4522,7 @@
         <v>0</v>
       </c>
       <c r="Y43" s="2">
-        <v>144789230</v>
+        <v>0</v>
       </c>
     </row>
     <row r="44" spans="1:25" x14ac:dyDescent="0.25">
@@ -4524,25 +4539,25 @@
         <v>3</v>
       </c>
       <c r="E44" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="F44" t="s">
-        <v>109</v>
+        <v>126</v>
       </c>
       <c r="G44" t="s">
-        <v>110</v>
+        <v>127</v>
       </c>
       <c r="H44" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="I44" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="J44" t="s">
         <v>9</v>
       </c>
       <c r="K44" s="2">
-        <v>316905738</v>
+        <v>12185731</v>
       </c>
       <c r="L44" s="2">
         <v>0</v>
@@ -4554,13 +4569,13 @@
         <v>0</v>
       </c>
       <c r="O44" s="2">
-        <v>0</v>
+        <v>-437763</v>
       </c>
       <c r="P44" s="2">
-        <v>0</v>
+        <v>-563094</v>
       </c>
       <c r="Q44" s="2">
-        <v>316905738</v>
+        <v>11184874</v>
       </c>
       <c r="R44" s="2">
         <v>0</v>
@@ -4601,13 +4616,13 @@
         <v>3</v>
       </c>
       <c r="E45" t="s">
-        <v>121</v>
+        <v>106</v>
       </c>
       <c r="F45" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G45" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H45" t="s">
         <v>130</v>
@@ -4619,7 +4634,7 @@
         <v>9</v>
       </c>
       <c r="K45" s="2">
-        <v>12185731</v>
+        <v>6064313</v>
       </c>
       <c r="L45" s="2">
         <v>0</v>
@@ -4631,13 +4646,13 @@
         <v>0</v>
       </c>
       <c r="O45" s="2">
-        <v>-437763</v>
+        <v>0</v>
       </c>
       <c r="P45" s="2">
-        <v>-563094</v>
+        <v>-731234</v>
       </c>
       <c r="Q45" s="2">
-        <v>11184874</v>
+        <v>5333079</v>
       </c>
       <c r="R45" s="2">
         <v>0</v>
@@ -4678,13 +4693,13 @@
         <v>3</v>
       </c>
       <c r="E46" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="F46" t="s">
-        <v>128</v>
+        <v>81</v>
       </c>
       <c r="G46" t="s">
-        <v>129</v>
+        <v>82</v>
       </c>
       <c r="H46" t="s">
         <v>132</v>
@@ -4696,10 +4711,10 @@
         <v>9</v>
       </c>
       <c r="K46" s="2">
-        <v>6064313</v>
+        <v>3404957</v>
       </c>
       <c r="L46" s="2">
-        <v>0</v>
+        <v>-286417</v>
       </c>
       <c r="M46" s="2">
         <v>0</v>
@@ -4711,10 +4726,10 @@
         <v>0</v>
       </c>
       <c r="P46" s="2">
-        <v>-731234</v>
+        <v>0</v>
       </c>
       <c r="Q46" s="2">
-        <v>5333079</v>
+        <v>3118540</v>
       </c>
       <c r="R46" s="2">
         <v>0</v>
@@ -4755,13 +4770,13 @@
         <v>3</v>
       </c>
       <c r="E47" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="F47" t="s">
-        <v>81</v>
+        <v>102</v>
       </c>
       <c r="G47" t="s">
-        <v>82</v>
+        <v>103</v>
       </c>
       <c r="H47" t="s">
         <v>134</v>
@@ -4773,10 +4788,10 @@
         <v>9</v>
       </c>
       <c r="K47" s="2">
-        <v>3404957</v>
+        <v>0</v>
       </c>
       <c r="L47" s="2">
-        <v>-286417</v>
+        <v>0</v>
       </c>
       <c r="M47" s="2">
         <v>0</v>
@@ -4788,10 +4803,10 @@
         <v>0</v>
       </c>
       <c r="P47" s="2">
-        <v>0</v>
+        <v>18628426</v>
       </c>
       <c r="Q47" s="2">
-        <v>3118540</v>
+        <v>18628426</v>
       </c>
       <c r="R47" s="2">
         <v>0</v>
@@ -4832,13 +4847,13 @@
         <v>3</v>
       </c>
       <c r="E48" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F48" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="G48" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="H48" t="s">
         <v>136</v>
@@ -4850,7 +4865,7 @@
         <v>9</v>
       </c>
       <c r="K48" s="2">
-        <v>0</v>
+        <v>54441960</v>
       </c>
       <c r="L48" s="2">
         <v>0</v>
@@ -4865,10 +4880,10 @@
         <v>0</v>
       </c>
       <c r="P48" s="2">
-        <v>18628426</v>
+        <v>0</v>
       </c>
       <c r="Q48" s="2">
-        <v>18628426</v>
+        <v>54441960</v>
       </c>
       <c r="R48" s="2">
         <v>0</v>
@@ -4909,7 +4924,7 @@
         <v>3</v>
       </c>
       <c r="E49" t="s">
-        <v>121</v>
+        <v>80</v>
       </c>
       <c r="F49" t="s">
         <v>81</v>
@@ -4927,25 +4942,25 @@
         <v>9</v>
       </c>
       <c r="K49" s="2">
-        <v>54441960</v>
+        <v>0</v>
       </c>
       <c r="L49" s="2">
-        <v>0</v>
+        <v>8553717</v>
       </c>
       <c r="M49" s="2">
-        <v>0</v>
+        <v>38598624</v>
       </c>
       <c r="N49" s="2">
         <v>0</v>
       </c>
       <c r="O49" s="2">
-        <v>0</v>
+        <v>47819368</v>
       </c>
       <c r="P49" s="2">
         <v>0</v>
       </c>
       <c r="Q49" s="2">
-        <v>54441960</v>
+        <v>94971709</v>
       </c>
       <c r="R49" s="2">
         <v>0</v>
@@ -4980,49 +4995,49 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>79</v>
+        <v>63</v>
       </c>
       <c r="D50" t="s">
         <v>3</v>
       </c>
       <c r="E50" t="s">
-        <v>80</v>
+        <v>140</v>
       </c>
       <c r="F50" t="s">
-        <v>81</v>
+        <v>65</v>
       </c>
       <c r="G50" t="s">
-        <v>82</v>
+        <v>66</v>
       </c>
       <c r="H50" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I50" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J50" t="s">
         <v>9</v>
       </c>
       <c r="K50" s="2">
-        <v>0</v>
+        <v>38394000</v>
       </c>
       <c r="L50" s="2">
-        <v>8553717</v>
+        <v>0</v>
       </c>
       <c r="M50" s="2">
-        <v>38598624</v>
+        <v>0</v>
       </c>
       <c r="N50" s="2">
         <v>0</v>
       </c>
       <c r="O50" s="2">
-        <v>47819368</v>
+        <v>0</v>
       </c>
       <c r="P50" s="2">
         <v>0</v>
       </c>
       <c r="Q50" s="2">
-        <v>94971709</v>
+        <v>38394000</v>
       </c>
       <c r="R50" s="2">
         <v>0</v>
@@ -5063,7 +5078,7 @@
         <v>3</v>
       </c>
       <c r="E51" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="F51" t="s">
         <v>65</v>
@@ -5081,10 +5096,10 @@
         <v>9</v>
       </c>
       <c r="K51" s="2">
-        <v>38394000</v>
+        <v>107244000</v>
       </c>
       <c r="L51" s="2">
-        <v>0</v>
+        <v>14874800</v>
       </c>
       <c r="M51" s="2">
         <v>0</v>
@@ -5099,7 +5114,7 @@
         <v>0</v>
       </c>
       <c r="Q51" s="2">
-        <v>38394000</v>
+        <v>122118800</v>
       </c>
       <c r="R51" s="2">
         <v>0</v>
@@ -5134,19 +5149,19 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="D52" t="s">
         <v>3</v>
       </c>
       <c r="E52" t="s">
-        <v>142</v>
+        <v>4</v>
       </c>
       <c r="F52" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="G52" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="H52" t="s">
         <v>145</v>
@@ -5158,10 +5173,10 @@
         <v>9</v>
       </c>
       <c r="K52" s="2">
-        <v>107244000</v>
+        <v>15683328</v>
       </c>
       <c r="L52" s="2">
-        <v>14874800</v>
+        <v>0</v>
       </c>
       <c r="M52" s="2">
         <v>0</v>
@@ -5176,7 +5191,7 @@
         <v>0</v>
       </c>
       <c r="Q52" s="2">
-        <v>122118800</v>
+        <v>15683328</v>
       </c>
       <c r="R52" s="2">
         <v>0</v>
@@ -5365,19 +5380,19 @@
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D55" t="s">
         <v>3</v>
       </c>
       <c r="E55" t="s">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="F55" t="s">
-        <v>43</v>
+        <v>102</v>
       </c>
       <c r="G55" t="s">
-        <v>44</v>
+        <v>103</v>
       </c>
       <c r="H55" t="s">
         <v>153</v>
@@ -5389,10 +5404,10 @@
         <v>9</v>
       </c>
       <c r="K55" s="2">
-        <v>4448736</v>
+        <v>0</v>
       </c>
       <c r="L55" s="2">
-        <v>0</v>
+        <v>21506679</v>
       </c>
       <c r="M55" s="2">
         <v>0</v>
@@ -5407,7 +5422,7 @@
         <v>0</v>
       </c>
       <c r="Q55" s="2">
-        <v>4448736</v>
+        <v>21506679</v>
       </c>
       <c r="R55" s="2">
         <v>0</v>
@@ -5442,19 +5457,19 @@
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D56" t="s">
         <v>3</v>
       </c>
       <c r="E56" t="s">
-        <v>108</v>
+        <v>4</v>
       </c>
       <c r="F56" t="s">
-        <v>104</v>
+        <v>43</v>
       </c>
       <c r="G56" t="s">
-        <v>105</v>
+        <v>44</v>
       </c>
       <c r="H56" t="s">
         <v>155</v>
@@ -5466,10 +5481,10 @@
         <v>9</v>
       </c>
       <c r="K56" s="2">
-        <v>0</v>
+        <v>201139200</v>
       </c>
       <c r="L56" s="2">
-        <v>21506679</v>
+        <v>0</v>
       </c>
       <c r="M56" s="2">
         <v>0</v>
@@ -5484,7 +5499,7 @@
         <v>0</v>
       </c>
       <c r="Q56" s="2">
-        <v>21506679</v>
+        <v>201139200</v>
       </c>
       <c r="R56" s="2">
         <v>0</v>
@@ -5528,10 +5543,10 @@
         <v>4</v>
       </c>
       <c r="F57" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="G57" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="H57" t="s">
         <v>157</v>
@@ -5543,7 +5558,7 @@
         <v>9</v>
       </c>
       <c r="K57" s="2">
-        <v>201139200</v>
+        <v>2565648</v>
       </c>
       <c r="L57" s="2">
         <v>0</v>
@@ -5561,7 +5576,7 @@
         <v>0</v>
       </c>
       <c r="Q57" s="2">
-        <v>201139200</v>
+        <v>2565648</v>
       </c>
       <c r="R57" s="2">
         <v>0</v>
@@ -5596,19 +5611,19 @@
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D58" t="s">
         <v>3</v>
       </c>
       <c r="E58" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F58" t="s">
-        <v>5</v>
+        <v>111</v>
       </c>
       <c r="G58" t="s">
-        <v>6</v>
+        <v>112</v>
       </c>
       <c r="H58" t="s">
         <v>159</v>
@@ -5620,7 +5635,7 @@
         <v>9</v>
       </c>
       <c r="K58" s="2">
-        <v>2565648</v>
+        <v>93045016</v>
       </c>
       <c r="L58" s="2">
         <v>0</v>
@@ -5638,7 +5653,7 @@
         <v>0</v>
       </c>
       <c r="Q58" s="2">
-        <v>2565648</v>
+        <v>93045016</v>
       </c>
       <c r="R58" s="2">
         <v>0</v>
@@ -5673,19 +5688,19 @@
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D59" t="s">
         <v>3</v>
       </c>
       <c r="E59" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F59" t="s">
-        <v>113</v>
+        <v>5</v>
       </c>
       <c r="G59" t="s">
-        <v>114</v>
+        <v>6</v>
       </c>
       <c r="H59" t="s">
         <v>161</v>
@@ -5697,7 +5712,7 @@
         <v>9</v>
       </c>
       <c r="K59" s="2">
-        <v>93045016</v>
+        <v>5769792</v>
       </c>
       <c r="L59" s="2">
         <v>0</v>
@@ -5715,7 +5730,7 @@
         <v>0</v>
       </c>
       <c r="Q59" s="2">
-        <v>93045016</v>
+        <v>5769792</v>
       </c>
       <c r="R59" s="2">
         <v>0</v>
@@ -5750,19 +5765,19 @@
         <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="D60" t="s">
         <v>3</v>
       </c>
       <c r="E60" t="s">
-        <v>4</v>
+        <v>140</v>
       </c>
       <c r="F60" t="s">
-        <v>5</v>
+        <v>65</v>
       </c>
       <c r="G60" t="s">
-        <v>6</v>
+        <v>66</v>
       </c>
       <c r="H60" t="s">
         <v>163</v>
@@ -5774,7 +5789,7 @@
         <v>9</v>
       </c>
       <c r="K60" s="2">
-        <v>5769792</v>
+        <v>3631392</v>
       </c>
       <c r="L60" s="2">
         <v>0</v>
@@ -5792,7 +5807,7 @@
         <v>0</v>
       </c>
       <c r="Q60" s="2">
-        <v>5769792</v>
+        <v>3631392</v>
       </c>
       <c r="R60" s="2">
         <v>0</v>
@@ -5827,19 +5842,19 @@
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="D61" t="s">
         <v>3</v>
       </c>
       <c r="E61" t="s">
-        <v>142</v>
+        <v>4</v>
       </c>
       <c r="F61" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="G61" t="s">
-        <v>66</v>
+        <v>50</v>
       </c>
       <c r="H61" t="s">
         <v>165</v>
@@ -5851,7 +5866,7 @@
         <v>9</v>
       </c>
       <c r="K61" s="2">
-        <v>3631392</v>
+        <v>303350184</v>
       </c>
       <c r="L61" s="2">
         <v>0</v>
@@ -5869,7 +5884,7 @@
         <v>0</v>
       </c>
       <c r="Q61" s="2">
-        <v>3631392</v>
+        <v>303350184</v>
       </c>
       <c r="R61" s="2">
         <v>0</v>
@@ -5904,19 +5919,19 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D62" t="s">
         <v>3</v>
       </c>
       <c r="E62" t="s">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="F62" t="s">
-        <v>49</v>
+        <v>102</v>
       </c>
       <c r="G62" t="s">
-        <v>50</v>
+        <v>103</v>
       </c>
       <c r="H62" t="s">
         <v>167</v>
@@ -5928,7 +5943,7 @@
         <v>9</v>
       </c>
       <c r="K62" s="2">
-        <v>303350184</v>
+        <v>11767702</v>
       </c>
       <c r="L62" s="2">
         <v>0</v>
@@ -5946,7 +5961,7 @@
         <v>0</v>
       </c>
       <c r="Q62" s="2">
-        <v>303350184</v>
+        <v>11767702</v>
       </c>
       <c r="R62" s="2">
         <v>0</v>
@@ -5987,13 +6002,13 @@
         <v>3</v>
       </c>
       <c r="E63" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F63" t="s">
-        <v>104</v>
+        <v>81</v>
       </c>
       <c r="G63" t="s">
-        <v>105</v>
+        <v>82</v>
       </c>
       <c r="H63" t="s">
         <v>169</v>
@@ -6005,7 +6020,7 @@
         <v>9</v>
       </c>
       <c r="K63" s="2">
-        <v>11767702</v>
+        <v>0</v>
       </c>
       <c r="L63" s="2">
         <v>0</v>
@@ -6020,10 +6035,10 @@
         <v>0</v>
       </c>
       <c r="P63" s="2">
-        <v>0</v>
+        <v>30207046</v>
       </c>
       <c r="Q63" s="2">
-        <v>11767702</v>
+        <v>30207046</v>
       </c>
       <c r="R63" s="2">
         <v>0</v>
@@ -6064,19 +6079,19 @@
         <v>3</v>
       </c>
       <c r="E64" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F64" t="s">
-        <v>81</v>
+        <v>171</v>
       </c>
       <c r="G64" t="s">
-        <v>82</v>
+        <v>172</v>
       </c>
       <c r="H64" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="I64" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="J64" t="s">
         <v>9</v>
@@ -6097,10 +6112,10 @@
         <v>0</v>
       </c>
       <c r="P64" s="2">
-        <v>30207046</v>
+        <v>8518911</v>
       </c>
       <c r="Q64" s="2">
-        <v>30207046</v>
+        <v>8518911</v>
       </c>
       <c r="R64" s="2">
         <v>0</v>
@@ -6135,31 +6150,31 @@
         <v>1</v>
       </c>
       <c r="C65" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D65" t="s">
         <v>3</v>
       </c>
       <c r="E65" t="s">
-        <v>108</v>
+        <v>4</v>
       </c>
       <c r="F65" t="s">
+        <v>5</v>
+      </c>
+      <c r="G65" t="s">
+        <v>6</v>
+      </c>
+      <c r="H65" t="s">
         <v>173</v>
       </c>
-      <c r="G65" t="s">
+      <c r="I65" t="s">
         <v>174</v>
       </c>
-      <c r="H65" t="s">
-        <v>171</v>
-      </c>
-      <c r="I65" t="s">
-        <v>172</v>
-      </c>
       <c r="J65" t="s">
         <v>9</v>
       </c>
       <c r="K65" s="2">
-        <v>0</v>
+        <v>172499760</v>
       </c>
       <c r="L65" s="2">
         <v>0</v>
@@ -6174,10 +6189,10 @@
         <v>0</v>
       </c>
       <c r="P65" s="2">
-        <v>8518911</v>
+        <v>0</v>
       </c>
       <c r="Q65" s="2">
-        <v>8518911</v>
+        <v>172499760</v>
       </c>
       <c r="R65" s="2">
         <v>0</v>
@@ -6212,19 +6227,19 @@
         <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D66" t="s">
         <v>3</v>
       </c>
       <c r="E66" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F66" t="s">
-        <v>5</v>
+        <v>102</v>
       </c>
       <c r="G66" t="s">
-        <v>6</v>
+        <v>103</v>
       </c>
       <c r="H66" t="s">
         <v>175</v>
@@ -6236,7 +6251,7 @@
         <v>9</v>
       </c>
       <c r="K66" s="2">
-        <v>172499760</v>
+        <v>14786158</v>
       </c>
       <c r="L66" s="2">
         <v>0</v>
@@ -6254,7 +6269,7 @@
         <v>0</v>
       </c>
       <c r="Q66" s="2">
-        <v>172499760</v>
+        <v>14786158</v>
       </c>
       <c r="R66" s="2">
         <v>0</v>
@@ -6289,19 +6304,19 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D67" t="s">
         <v>3</v>
       </c>
       <c r="E67" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F67" t="s">
-        <v>104</v>
+        <v>15</v>
       </c>
       <c r="G67" t="s">
-        <v>105</v>
+        <v>16</v>
       </c>
       <c r="H67" t="s">
         <v>177</v>
@@ -6313,7 +6328,7 @@
         <v>9</v>
       </c>
       <c r="K67" s="2">
-        <v>14786158</v>
+        <v>48819936</v>
       </c>
       <c r="L67" s="2">
         <v>0</v>
@@ -6331,7 +6346,7 @@
         <v>0</v>
       </c>
       <c r="Q67" s="2">
-        <v>14786158</v>
+        <v>48819936</v>
       </c>
       <c r="R67" s="2">
         <v>0</v>
@@ -6375,10 +6390,10 @@
         <v>4</v>
       </c>
       <c r="F68" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G68" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="H68" t="s">
         <v>179</v>
@@ -6390,10 +6405,10 @@
         <v>9</v>
       </c>
       <c r="K68" s="2">
-        <v>48819936</v>
+        <v>49120000</v>
       </c>
       <c r="L68" s="2">
-        <v>0</v>
+        <v>245569000</v>
       </c>
       <c r="M68" s="2">
         <v>0</v>
@@ -6408,7 +6423,7 @@
         <v>0</v>
       </c>
       <c r="Q68" s="2">
-        <v>48819936</v>
+        <v>294689000</v>
       </c>
       <c r="R68" s="2">
         <v>0</v>
@@ -6452,25 +6467,25 @@
         <v>4</v>
       </c>
       <c r="F69" t="s">
-        <v>19</v>
+        <v>181</v>
       </c>
       <c r="G69" t="s">
-        <v>20</v>
+        <v>182</v>
       </c>
       <c r="H69" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="I69" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="J69" t="s">
         <v>9</v>
       </c>
       <c r="K69" s="2">
-        <v>49120000</v>
+        <v>28691280</v>
       </c>
       <c r="L69" s="2">
-        <v>245569000</v>
+        <v>35977392</v>
       </c>
       <c r="M69" s="2">
         <v>0</v>
@@ -6485,7 +6500,7 @@
         <v>0</v>
       </c>
       <c r="Q69" s="2">
-        <v>294689000</v>
+        <v>64668672</v>
       </c>
       <c r="R69" s="2">
         <v>0</v>
@@ -6529,10 +6544,10 @@
         <v>4</v>
       </c>
       <c r="F70" t="s">
-        <v>183</v>
+        <v>49</v>
       </c>
       <c r="G70" t="s">
-        <v>184</v>
+        <v>50</v>
       </c>
       <c r="H70" t="s">
         <v>185</v>
@@ -6544,10 +6559,10 @@
         <v>9</v>
       </c>
       <c r="K70" s="2">
-        <v>28691280</v>
+        <v>555141168</v>
       </c>
       <c r="L70" s="2">
-        <v>35977392</v>
+        <v>0</v>
       </c>
       <c r="M70" s="2">
         <v>0</v>
@@ -6562,7 +6577,7 @@
         <v>0</v>
       </c>
       <c r="Q70" s="2">
-        <v>64668672</v>
+        <v>555141168</v>
       </c>
       <c r="R70" s="2">
         <v>0</v>
@@ -6597,19 +6612,19 @@
         <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D71" t="s">
         <v>3</v>
       </c>
       <c r="E71" t="s">
-        <v>4</v>
+        <v>106</v>
       </c>
       <c r="F71" t="s">
-        <v>49</v>
+        <v>107</v>
       </c>
       <c r="G71" t="s">
-        <v>50</v>
+        <v>108</v>
       </c>
       <c r="H71" t="s">
         <v>187</v>
@@ -6621,25 +6636,25 @@
         <v>9</v>
       </c>
       <c r="K71" s="2">
-        <v>555141168</v>
+        <v>15037055</v>
       </c>
       <c r="L71" s="2">
-        <v>0</v>
+        <v>10235715</v>
       </c>
       <c r="M71" s="2">
-        <v>0</v>
+        <v>8519043</v>
       </c>
       <c r="N71" s="2">
         <v>0</v>
       </c>
       <c r="O71" s="2">
-        <v>0</v>
+        <v>29470499</v>
       </c>
       <c r="P71" s="2">
         <v>0</v>
       </c>
       <c r="Q71" s="2">
-        <v>555141168</v>
+        <v>63262312</v>
       </c>
       <c r="R71" s="2">
         <v>0</v>
@@ -6680,13 +6695,13 @@
         <v>3</v>
       </c>
       <c r="E72" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F72" t="s">
-        <v>109</v>
+        <v>81</v>
       </c>
       <c r="G72" t="s">
-        <v>110</v>
+        <v>82</v>
       </c>
       <c r="H72" t="s">
         <v>189</v>
@@ -6698,25 +6713,25 @@
         <v>9</v>
       </c>
       <c r="K72" s="2">
-        <v>15037055</v>
+        <v>60080164</v>
       </c>
       <c r="L72" s="2">
-        <v>10235715</v>
+        <v>0</v>
       </c>
       <c r="M72" s="2">
-        <v>8519043</v>
+        <v>0</v>
       </c>
       <c r="N72" s="2">
         <v>0</v>
       </c>
       <c r="O72" s="2">
-        <v>29470499</v>
+        <v>0</v>
       </c>
       <c r="P72" s="2">
         <v>0</v>
       </c>
       <c r="Q72" s="2">
-        <v>63262312</v>
+        <v>60080164</v>
       </c>
       <c r="R72" s="2">
         <v>0</v>
@@ -6751,19 +6766,19 @@
         <v>1</v>
       </c>
       <c r="C73" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D73" t="s">
         <v>3</v>
       </c>
       <c r="E73" t="s">
-        <v>108</v>
+        <v>4</v>
       </c>
       <c r="F73" t="s">
-        <v>81</v>
+        <v>15</v>
       </c>
       <c r="G73" t="s">
-        <v>82</v>
+        <v>16</v>
       </c>
       <c r="H73" t="s">
         <v>191</v>
@@ -6775,7 +6790,7 @@
         <v>9</v>
       </c>
       <c r="K73" s="2">
-        <v>60080164</v>
+        <v>24122016</v>
       </c>
       <c r="L73" s="2">
         <v>0</v>
@@ -6793,7 +6808,7 @@
         <v>0</v>
       </c>
       <c r="Q73" s="2">
-        <v>60080164</v>
+        <v>24122016</v>
       </c>
       <c r="R73" s="2">
         <v>0</v>
@@ -6828,19 +6843,19 @@
         <v>1</v>
       </c>
       <c r="C74" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D74" t="s">
         <v>3</v>
       </c>
       <c r="E74" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F74" t="s">
-        <v>15</v>
+        <v>126</v>
       </c>
       <c r="G74" t="s">
-        <v>16</v>
+        <v>127</v>
       </c>
       <c r="H74" t="s">
         <v>193</v>
@@ -6852,7 +6867,7 @@
         <v>9</v>
       </c>
       <c r="K74" s="2">
-        <v>24122016</v>
+        <v>47527794</v>
       </c>
       <c r="L74" s="2">
         <v>0</v>
@@ -6870,7 +6885,7 @@
         <v>0</v>
       </c>
       <c r="Q74" s="2">
-        <v>24122016</v>
+        <v>47527794</v>
       </c>
       <c r="R74" s="2">
         <v>0</v>
@@ -6911,13 +6926,13 @@
         <v>3</v>
       </c>
       <c r="E75" t="s">
-        <v>80</v>
+        <v>119</v>
       </c>
       <c r="F75" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="G75" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="H75" t="s">
         <v>195</v>
@@ -6929,7 +6944,7 @@
         <v>9</v>
       </c>
       <c r="K75" s="2">
-        <v>47527794</v>
+        <v>19090076</v>
       </c>
       <c r="L75" s="2">
         <v>0</v>
@@ -6947,7 +6962,7 @@
         <v>0</v>
       </c>
       <c r="Q75" s="2">
-        <v>47527794</v>
+        <v>19090076</v>
       </c>
       <c r="R75" s="2">
         <v>0</v>
@@ -6982,19 +6997,19 @@
         <v>1</v>
       </c>
       <c r="C76" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D76" t="s">
         <v>3</v>
       </c>
       <c r="E76" t="s">
-        <v>121</v>
+        <v>4</v>
       </c>
       <c r="F76" t="s">
-        <v>128</v>
+        <v>43</v>
       </c>
       <c r="G76" t="s">
-        <v>129</v>
+        <v>44</v>
       </c>
       <c r="H76" t="s">
         <v>197</v>
@@ -7006,7 +7021,7 @@
         <v>9</v>
       </c>
       <c r="K76" s="2">
-        <v>19090076</v>
+        <v>768791770</v>
       </c>
       <c r="L76" s="2">
         <v>0</v>
@@ -7024,7 +7039,7 @@
         <v>0</v>
       </c>
       <c r="Q76" s="2">
-        <v>19090076</v>
+        <v>768791770</v>
       </c>
       <c r="R76" s="2">
         <v>0</v>
@@ -7059,19 +7074,19 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D77" t="s">
         <v>3</v>
       </c>
       <c r="E77" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F77" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
       <c r="G77" t="s">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="H77" t="s">
         <v>199</v>
@@ -7083,7 +7098,7 @@
         <v>9</v>
       </c>
       <c r="K77" s="2">
-        <v>768791770</v>
+        <v>18664603</v>
       </c>
       <c r="L77" s="2">
         <v>0</v>
@@ -7092,7 +7107,7 @@
         <v>0</v>
       </c>
       <c r="N77" s="2">
-        <v>0</v>
+        <v>1764004</v>
       </c>
       <c r="O77" s="2">
         <v>0</v>
@@ -7101,7 +7116,7 @@
         <v>0</v>
       </c>
       <c r="Q77" s="2">
-        <v>768791770</v>
+        <v>20428607</v>
       </c>
       <c r="R77" s="2">
         <v>0</v>
@@ -7136,19 +7151,19 @@
         <v>1</v>
       </c>
       <c r="C78" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D78" t="s">
         <v>3</v>
       </c>
       <c r="E78" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F78" t="s">
-        <v>81</v>
+        <v>10</v>
       </c>
       <c r="G78" t="s">
-        <v>82</v>
+        <v>11</v>
       </c>
       <c r="H78" t="s">
         <v>201</v>
@@ -7160,16 +7175,16 @@
         <v>9</v>
       </c>
       <c r="K78" s="2">
-        <v>18664603</v>
+        <v>242095176</v>
       </c>
       <c r="L78" s="2">
-        <v>0</v>
+        <v>132300648</v>
       </c>
       <c r="M78" s="2">
         <v>0</v>
       </c>
       <c r="N78" s="2">
-        <v>1764004</v>
+        <v>0</v>
       </c>
       <c r="O78" s="2">
         <v>0</v>
@@ -7178,7 +7193,7 @@
         <v>0</v>
       </c>
       <c r="Q78" s="2">
-        <v>20428607</v>
+        <v>374395824</v>
       </c>
       <c r="R78" s="2">
         <v>0</v>
@@ -7187,7 +7202,7 @@
         <v>0</v>
       </c>
       <c r="T78" s="2">
-        <v>0</v>
+        <v>52586280</v>
       </c>
       <c r="U78" s="2">
         <v>0</v>
@@ -7202,7 +7217,7 @@
         <v>0</v>
       </c>
       <c r="Y78" s="2">
-        <v>0</v>
+        <v>52586280</v>
       </c>
     </row>
     <row r="79" spans="1:25" x14ac:dyDescent="0.25">
@@ -7222,10 +7237,10 @@
         <v>4</v>
       </c>
       <c r="F79" t="s">
-        <v>10</v>
+        <v>181</v>
       </c>
       <c r="G79" t="s">
-        <v>11</v>
+        <v>182</v>
       </c>
       <c r="H79" t="s">
         <v>203</v>
@@ -7237,10 +7252,10 @@
         <v>9</v>
       </c>
       <c r="K79" s="2">
-        <v>242095176</v>
+        <v>0</v>
       </c>
       <c r="L79" s="2">
-        <v>132300648</v>
+        <v>64740000</v>
       </c>
       <c r="M79" s="2">
         <v>0</v>
@@ -7255,7 +7270,7 @@
         <v>0</v>
       </c>
       <c r="Q79" s="2">
-        <v>374395824</v>
+        <v>64740000</v>
       </c>
       <c r="R79" s="2">
         <v>0</v>
@@ -7264,7 +7279,7 @@
         <v>0</v>
       </c>
       <c r="T79" s="2">
-        <v>52586280</v>
+        <v>0</v>
       </c>
       <c r="U79" s="2">
         <v>0</v>
@@ -7279,7 +7294,7 @@
         <v>0</v>
       </c>
       <c r="Y79" s="2">
-        <v>52586280</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:25" x14ac:dyDescent="0.25">
@@ -7290,19 +7305,19 @@
         <v>1</v>
       </c>
       <c r="C80" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D80" t="s">
         <v>3</v>
       </c>
       <c r="E80" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F80" t="s">
-        <v>183</v>
+        <v>126</v>
       </c>
       <c r="G80" t="s">
-        <v>184</v>
+        <v>127</v>
       </c>
       <c r="H80" t="s">
         <v>205</v>
@@ -7317,13 +7332,13 @@
         <v>0</v>
       </c>
       <c r="L80" s="2">
-        <v>64740000</v>
+        <v>45331549</v>
       </c>
       <c r="M80" s="2">
         <v>0</v>
       </c>
       <c r="N80" s="2">
-        <v>0</v>
+        <v>47387128</v>
       </c>
       <c r="O80" s="2">
         <v>0</v>
@@ -7332,7 +7347,7 @@
         <v>0</v>
       </c>
       <c r="Q80" s="2">
-        <v>64740000</v>
+        <v>92718677</v>
       </c>
       <c r="R80" s="2">
         <v>0</v>
@@ -7376,10 +7391,10 @@
         <v>80</v>
       </c>
       <c r="F81" t="s">
-        <v>128</v>
+        <v>149</v>
       </c>
       <c r="G81" t="s">
-        <v>129</v>
+        <v>150</v>
       </c>
       <c r="H81" t="s">
         <v>207</v>
@@ -7391,16 +7406,16 @@
         <v>9</v>
       </c>
       <c r="K81" s="2">
-        <v>0</v>
+        <v>115727621</v>
       </c>
       <c r="L81" s="2">
-        <v>45331549</v>
+        <v>0</v>
       </c>
       <c r="M81" s="2">
         <v>0</v>
       </c>
       <c r="N81" s="2">
-        <v>47387128</v>
+        <v>0</v>
       </c>
       <c r="O81" s="2">
         <v>0</v>
@@ -7409,7 +7424,7 @@
         <v>0</v>
       </c>
       <c r="Q81" s="2">
-        <v>92718677</v>
+        <v>115727621</v>
       </c>
       <c r="R81" s="2">
         <v>0</v>
@@ -7444,31 +7459,31 @@
         <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D82" t="s">
         <v>3</v>
       </c>
       <c r="E82" t="s">
-        <v>80</v>
+        <v>209</v>
       </c>
       <c r="F82" t="s">
-        <v>149</v>
+        <v>43</v>
       </c>
       <c r="G82" t="s">
-        <v>150</v>
+        <v>44</v>
       </c>
       <c r="H82" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I82" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="J82" t="s">
         <v>9</v>
       </c>
       <c r="K82" s="2">
-        <v>115727621</v>
+        <v>151200000</v>
       </c>
       <c r="L82" s="2">
         <v>0</v>
@@ -7486,7 +7501,7 @@
         <v>0</v>
       </c>
       <c r="Q82" s="2">
-        <v>115727621</v>
+        <v>151200000</v>
       </c>
       <c r="R82" s="2">
         <v>0</v>
@@ -7521,19 +7536,19 @@
         <v>1</v>
       </c>
       <c r="C83" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D83" t="s">
         <v>3</v>
       </c>
       <c r="E83" t="s">
-        <v>211</v>
+        <v>85</v>
       </c>
       <c r="F83" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
       <c r="G83" t="s">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="H83" t="s">
         <v>212</v>
@@ -7545,10 +7560,10 @@
         <v>9</v>
       </c>
       <c r="K83" s="2">
-        <v>151200000</v>
+        <v>1533149</v>
       </c>
       <c r="L83" s="2">
-        <v>0</v>
+        <v>709159</v>
       </c>
       <c r="M83" s="2">
         <v>0</v>
@@ -7563,10 +7578,10 @@
         <v>0</v>
       </c>
       <c r="Q83" s="2">
-        <v>151200000</v>
+        <v>2242308</v>
       </c>
       <c r="R83" s="2">
-        <v>0</v>
+        <v>839744</v>
       </c>
       <c r="S83" s="2">
         <v>0</v>
@@ -7587,7 +7602,7 @@
         <v>0</v>
       </c>
       <c r="Y83" s="2">
-        <v>0</v>
+        <v>839744</v>
       </c>
     </row>
     <row r="84" spans="1:25" x14ac:dyDescent="0.25">
@@ -7604,13 +7619,13 @@
         <v>3</v>
       </c>
       <c r="E84" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F84" t="s">
-        <v>81</v>
+        <v>149</v>
       </c>
       <c r="G84" t="s">
-        <v>82</v>
+        <v>150</v>
       </c>
       <c r="H84" t="s">
         <v>214</v>
@@ -7622,10 +7637,10 @@
         <v>9</v>
       </c>
       <c r="K84" s="2">
-        <v>1533149</v>
+        <v>-302587</v>
       </c>
       <c r="L84" s="2">
-        <v>709159</v>
+        <v>0</v>
       </c>
       <c r="M84" s="2">
         <v>0</v>
@@ -7640,10 +7655,10 @@
         <v>0</v>
       </c>
       <c r="Q84" s="2">
-        <v>2242308</v>
+        <v>-302587</v>
       </c>
       <c r="R84" s="2">
-        <v>839744</v>
+        <v>0</v>
       </c>
       <c r="S84" s="2">
         <v>0</v>
@@ -7664,7 +7679,7 @@
         <v>0</v>
       </c>
       <c r="Y84" s="2">
-        <v>839744</v>
+        <v>0</v>
       </c>
     </row>
     <row r="85" spans="1:25" x14ac:dyDescent="0.25">
@@ -7675,31 +7690,31 @@
         <v>1</v>
       </c>
       <c r="C85" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D85" t="s">
         <v>3</v>
       </c>
       <c r="E85" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F85" t="s">
-        <v>149</v>
+        <v>216</v>
       </c>
       <c r="G85" t="s">
-        <v>150</v>
+        <v>3</v>
       </c>
       <c r="H85" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="I85" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="J85" t="s">
         <v>9</v>
       </c>
       <c r="K85" s="2">
-        <v>-302587</v>
+        <v>1662768</v>
       </c>
       <c r="L85" s="2">
         <v>0</v>
@@ -7717,7 +7732,7 @@
         <v>0</v>
       </c>
       <c r="Q85" s="2">
-        <v>-302587</v>
+        <v>1662768</v>
       </c>
       <c r="R85" s="2">
         <v>0</v>
@@ -7761,16 +7776,16 @@
         <v>80</v>
       </c>
       <c r="F86" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G86" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H86" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="I86" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="J86" t="s">
         <v>9</v>
@@ -7844,10 +7859,10 @@
         <v>16</v>
       </c>
       <c r="H87" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I87" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="J87" t="s">
         <v>9</v>
@@ -7915,16 +7930,16 @@
         <v>80</v>
       </c>
       <c r="F88" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="G88" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="H88" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="I88" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="J88" t="s">
         <v>9</v>
@@ -7989,19 +8004,19 @@
         <v>3</v>
       </c>
       <c r="E89" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F89" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="G89" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="H89" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="I89" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="J89" t="s">
         <v>9</v>
@@ -8066,7 +8081,7 @@
         <v>3</v>
       </c>
       <c r="E90" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F90" t="s">
         <v>88</v>
@@ -8075,10 +8090,10 @@
         <v>89</v>
       </c>
       <c r="H90" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="I90" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="J90" t="s">
         <v>9</v>
@@ -8143,7 +8158,7 @@
         <v>3</v>
       </c>
       <c r="E91" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F91" t="s">
         <v>81</v>
@@ -8152,10 +8167,10 @@
         <v>82</v>
       </c>
       <c r="H91" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="I91" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="J91" t="s">
         <v>9</v>
@@ -8220,7 +8235,7 @@
         <v>3</v>
       </c>
       <c r="E92" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F92" t="s">
         <v>81</v>
@@ -8229,10 +8244,10 @@
         <v>82</v>
       </c>
       <c r="H92" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="I92" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="J92" t="s">
         <v>9</v>
@@ -8306,10 +8321,10 @@
         <v>82</v>
       </c>
       <c r="H93" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="I93" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="J93" t="s">
         <v>9</v>
@@ -8383,16 +8398,16 @@
         <v>6</v>
       </c>
       <c r="H94" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="I94" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="J94" t="s">
         <v>9</v>
       </c>
       <c r="K94" s="2">
-        <v>37748160</v>
+        <v>10069920</v>
       </c>
       <c r="L94" s="2">
         <v>0</v>
@@ -8410,13 +8425,13 @@
         <v>0</v>
       </c>
       <c r="Q94" s="2">
-        <v>37748160</v>
+        <v>10069920</v>
       </c>
       <c r="R94" s="2">
         <v>0</v>
       </c>
       <c r="S94" s="2">
-        <v>37748160</v>
+        <v>10069920</v>
       </c>
       <c r="T94" s="2">
         <v>0</v>
@@ -8434,7 +8449,7 @@
         <v>0</v>
       </c>
       <c r="Y94" s="2">
-        <v>37748160</v>
+        <v>10069920</v>
       </c>
     </row>
     <row r="95" spans="1:25" x14ac:dyDescent="0.25">
@@ -8454,22 +8469,22 @@
         <v>4</v>
       </c>
       <c r="F95" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G95" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H95" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="I95" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="J95" t="s">
         <v>9</v>
       </c>
       <c r="K95" s="2">
-        <v>11043605</v>
+        <v>4448736</v>
       </c>
       <c r="L95" s="2">
         <v>0</v>
@@ -8487,13 +8502,13 @@
         <v>0</v>
       </c>
       <c r="Q95" s="2">
-        <v>11043605</v>
+        <v>4448736</v>
       </c>
       <c r="R95" s="2">
         <v>0</v>
       </c>
       <c r="S95" s="2">
-        <v>11043605</v>
+        <v>4448736</v>
       </c>
       <c r="T95" s="2">
         <v>0</v>
@@ -8511,7 +8526,7 @@
         <v>0</v>
       </c>
       <c r="Y95" s="2">
-        <v>11043605</v>
+        <v>4448736</v>
       </c>
     </row>
     <row r="96" spans="1:25" x14ac:dyDescent="0.25">
@@ -8531,22 +8546,22 @@
         <v>4</v>
       </c>
       <c r="F96" t="s">
-        <v>43</v>
+        <v>5</v>
       </c>
       <c r="G96" t="s">
-        <v>44</v>
+        <v>6</v>
       </c>
       <c r="H96" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="I96" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J96" t="s">
         <v>9</v>
       </c>
       <c r="K96" s="2">
-        <v>14376960</v>
+        <v>37748160</v>
       </c>
       <c r="L96" s="2">
         <v>0</v>
@@ -8564,13 +8579,13 @@
         <v>0</v>
       </c>
       <c r="Q96" s="2">
-        <v>14376960</v>
+        <v>37748160</v>
       </c>
       <c r="R96" s="2">
         <v>0</v>
       </c>
       <c r="S96" s="2">
-        <v>14376960</v>
+        <v>37748160</v>
       </c>
       <c r="T96" s="2">
         <v>0</v>
@@ -8588,7 +8603,7 @@
         <v>0</v>
       </c>
       <c r="Y96" s="2">
-        <v>14376960</v>
+        <v>37748160</v>
       </c>
     </row>
     <row r="97" spans="1:25" x14ac:dyDescent="0.25">
@@ -8608,68 +8623,299 @@
         <v>4</v>
       </c>
       <c r="F97" t="s">
+        <v>49</v>
+      </c>
+      <c r="G97" t="s">
+        <v>50</v>
+      </c>
+      <c r="H97" t="s">
+        <v>242</v>
+      </c>
+      <c r="I97" t="s">
+        <v>243</v>
+      </c>
+      <c r="J97" t="s">
+        <v>9</v>
+      </c>
+      <c r="K97" s="2">
+        <v>11043605</v>
+      </c>
+      <c r="L97" s="2">
+        <v>0</v>
+      </c>
+      <c r="M97" s="2">
+        <v>0</v>
+      </c>
+      <c r="N97" s="2">
+        <v>0</v>
+      </c>
+      <c r="O97" s="2">
+        <v>0</v>
+      </c>
+      <c r="P97" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q97" s="2">
+        <v>11043605</v>
+      </c>
+      <c r="R97" s="2">
+        <v>0</v>
+      </c>
+      <c r="S97" s="2">
+        <v>11043605</v>
+      </c>
+      <c r="T97" s="2">
+        <v>0</v>
+      </c>
+      <c r="U97" s="2">
+        <v>0</v>
+      </c>
+      <c r="V97" s="2">
+        <v>0</v>
+      </c>
+      <c r="W97" s="2">
+        <v>0</v>
+      </c>
+      <c r="X97" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y97" s="2">
+        <v>11043605</v>
+      </c>
+    </row>
+    <row r="98" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>0</v>
+      </c>
+      <c r="B98" t="s">
+        <v>1</v>
+      </c>
+      <c r="C98" t="s">
+        <v>2</v>
+      </c>
+      <c r="D98" t="s">
+        <v>3</v>
+      </c>
+      <c r="E98" t="s">
+        <v>4</v>
+      </c>
+      <c r="F98" t="s">
+        <v>43</v>
+      </c>
+      <c r="G98" t="s">
+        <v>44</v>
+      </c>
+      <c r="H98" t="s">
+        <v>244</v>
+      </c>
+      <c r="I98" t="s">
+        <v>245</v>
+      </c>
+      <c r="J98" t="s">
+        <v>9</v>
+      </c>
+      <c r="K98" s="2">
+        <v>14376960</v>
+      </c>
+      <c r="L98" s="2">
+        <v>0</v>
+      </c>
+      <c r="M98" s="2">
+        <v>0</v>
+      </c>
+      <c r="N98" s="2">
+        <v>0</v>
+      </c>
+      <c r="O98" s="2">
+        <v>0</v>
+      </c>
+      <c r="P98" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q98" s="2">
+        <v>14376960</v>
+      </c>
+      <c r="R98" s="2">
+        <v>0</v>
+      </c>
+      <c r="S98" s="2">
+        <v>14376960</v>
+      </c>
+      <c r="T98" s="2">
+        <v>0</v>
+      </c>
+      <c r="U98" s="2">
+        <v>0</v>
+      </c>
+      <c r="V98" s="2">
+        <v>0</v>
+      </c>
+      <c r="W98" s="2">
+        <v>0</v>
+      </c>
+      <c r="X98" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y98" s="2">
+        <v>14376960</v>
+      </c>
+    </row>
+    <row r="99" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>0</v>
+      </c>
+      <c r="B99" t="s">
+        <v>1</v>
+      </c>
+      <c r="C99" t="s">
+        <v>2</v>
+      </c>
+      <c r="D99" t="s">
+        <v>3</v>
+      </c>
+      <c r="E99" t="s">
+        <v>4</v>
+      </c>
+      <c r="F99" t="s">
         <v>5</v>
       </c>
-      <c r="G97" t="s">
+      <c r="G99" t="s">
         <v>6</v>
       </c>
-      <c r="H97" t="s">
-        <v>241</v>
-      </c>
-      <c r="I97" t="s">
-        <v>242</v>
-      </c>
-      <c r="J97" t="s">
-        <v>9</v>
-      </c>
-      <c r="K97" s="2">
+      <c r="H99" t="s">
+        <v>246</v>
+      </c>
+      <c r="I99" t="s">
+        <v>247</v>
+      </c>
+      <c r="J99" t="s">
+        <v>9</v>
+      </c>
+      <c r="K99" s="2">
         <v>1987200</v>
       </c>
-      <c r="L97" s="2">
-        <v>0</v>
-      </c>
-      <c r="M97" s="2">
-        <v>0</v>
-      </c>
-      <c r="N97" s="2">
-        <v>0</v>
-      </c>
-      <c r="O97" s="2">
-        <v>0</v>
-      </c>
-      <c r="P97" s="2">
-        <v>0</v>
-      </c>
-      <c r="Q97" s="2">
+      <c r="L99" s="2">
+        <v>0</v>
+      </c>
+      <c r="M99" s="2">
+        <v>0</v>
+      </c>
+      <c r="N99" s="2">
+        <v>0</v>
+      </c>
+      <c r="O99" s="2">
+        <v>0</v>
+      </c>
+      <c r="P99" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q99" s="2">
         <v>1987200</v>
       </c>
-      <c r="R97" s="2">
-        <v>0</v>
-      </c>
-      <c r="S97" s="2">
+      <c r="R99" s="2">
+        <v>0</v>
+      </c>
+      <c r="S99" s="2">
         <v>1987200</v>
       </c>
-      <c r="T97" s="2">
-        <v>0</v>
-      </c>
-      <c r="U97" s="2">
-        <v>0</v>
-      </c>
-      <c r="V97" s="2">
-        <v>0</v>
-      </c>
-      <c r="W97" s="2">
-        <v>0</v>
-      </c>
-      <c r="X97" s="2">
-        <v>0</v>
-      </c>
-      <c r="Y97" s="2">
+      <c r="T99" s="2">
+        <v>0</v>
+      </c>
+      <c r="U99" s="2">
+        <v>0</v>
+      </c>
+      <c r="V99" s="2">
+        <v>0</v>
+      </c>
+      <c r="W99" s="2">
+        <v>0</v>
+      </c>
+      <c r="X99" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y99" s="2">
         <v>1987200</v>
       </c>
     </row>
+    <row r="100" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>0</v>
+      </c>
+      <c r="B100" t="s">
+        <v>1</v>
+      </c>
+      <c r="C100" t="s">
+        <v>2</v>
+      </c>
+      <c r="D100" t="s">
+        <v>3</v>
+      </c>
+      <c r="E100" t="s">
+        <v>80</v>
+      </c>
+      <c r="F100" t="s">
+        <v>216</v>
+      </c>
+      <c r="G100" t="s">
+        <v>3</v>
+      </c>
+      <c r="H100" t="s">
+        <v>83</v>
+      </c>
+      <c r="I100" t="s">
+        <v>84</v>
+      </c>
+      <c r="J100" t="s">
+        <v>9</v>
+      </c>
+      <c r="K100" s="2">
+        <v>600480</v>
+      </c>
+      <c r="L100" s="2">
+        <v>0</v>
+      </c>
+      <c r="M100" s="2">
+        <v>0</v>
+      </c>
+      <c r="N100" s="2">
+        <v>0</v>
+      </c>
+      <c r="O100" s="2">
+        <v>0</v>
+      </c>
+      <c r="P100" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q100" s="2">
+        <v>600480</v>
+      </c>
+      <c r="R100" s="2">
+        <v>0</v>
+      </c>
+      <c r="S100" s="2">
+        <v>600480</v>
+      </c>
+      <c r="T100" s="2">
+        <v>0</v>
+      </c>
+      <c r="U100" s="2">
+        <v>0</v>
+      </c>
+      <c r="V100" s="2">
+        <v>0</v>
+      </c>
+      <c r="W100" s="2">
+        <v>0</v>
+      </c>
+      <c r="X100" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y100" s="2">
+        <v>600480</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y97"/>
+  <autoFilter ref="A1:Y100"/>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter alignWithMargins="0"/>

</xml_diff>

<commit_message>
chore(core): clean upload service temporary files
</commit_message>
<xml_diff>
--- a/demodata/ZRFI005.XLSX
+++ b/demodata/ZRFI005.XLSX
@@ -15,14 +15,14 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Y$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$Y$103</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1015" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1045" uniqueCount="279">
   <si>
     <t>1000</t>
   </si>
@@ -300,6 +300,12 @@
     <t>CÔNG TY TNHH SX XNK THƯƠNG MẠI SÁNG</t>
   </si>
   <si>
+    <t>1200000548</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH DAIGAKU (VIỆT NAM)</t>
+  </si>
+  <si>
     <t>1200000560</t>
   </si>
   <si>
@@ -318,6 +324,12 @@
     <t>CÔNG TY CP XÂY DỰNG KIẾN TRÚC AA TÂY NINH</t>
   </si>
   <si>
+    <t>1200000769</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN KIM MỘC</t>
+  </si>
+  <si>
     <t>1200000786</t>
   </si>
   <si>
@@ -459,313 +471,319 @@
     <t>CÔNG TY TNHH THƯƠNG MẠI DỊCH VỤ XÂY DỰNG VÀ CÔNG NGHỆ SÀN SƠN PHÁT</t>
   </si>
   <si>
+    <t>1200000903</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH CÔNG NGHIỆP NHÀ XANH</t>
+  </si>
+  <si>
+    <t>10811780</t>
+  </si>
+  <si>
+    <t>TẠ DUY HÀ</t>
+  </si>
+  <si>
+    <t>1200000904</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH BẢO LÂM</t>
+  </si>
+  <si>
+    <t>1200000935</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN HỆ THỐNG SIÊU THỊ SƠN</t>
+  </si>
+  <si>
+    <t>1200000949</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN BAO BÌ IN KIM LOẠI THẾ KỶ</t>
+  </si>
+  <si>
+    <t>1200000963</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH CƠ KHÍ XÂY DỰNG VIỆT THẮNG</t>
+  </si>
+  <si>
+    <t>1200000971</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ SƠN ANH TÚ</t>
+  </si>
+  <si>
+    <t>1200000973</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH AN THỊNH FURNITURE</t>
+  </si>
+  <si>
+    <t>1200000992</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH DV KT AN TÂM PHÁT</t>
+  </si>
+  <si>
+    <t>1200001011</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN ĐÔNG NGÔ MANUFACTURER</t>
+  </si>
+  <si>
+    <t>1200001023</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI - DỊCH VỤ - XÂY DỰNG MAI TÂM</t>
+  </si>
+  <si>
+    <t>1200001029</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH TRANG TRÍ NỘI THẤT PHONG THẢO</t>
+  </si>
+  <si>
+    <t>10400773</t>
+  </si>
+  <si>
+    <t>VŨ ANH HAI</t>
+  </si>
+  <si>
+    <t>1200001038</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH PHÚ MỸ THĂNG</t>
+  </si>
+  <si>
+    <t>1200001041</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI XÂY DỰNG THIÊN PHÚ DECOR</t>
+  </si>
+  <si>
+    <t>1200001042</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH KIẾN TRÚC GỖ BỌC ĐÔ</t>
+  </si>
+  <si>
+    <t>1200001051</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH VINAWOOD</t>
+  </si>
+  <si>
+    <t>10999776</t>
+  </si>
+  <si>
+    <t>ĐẶNG VĂN CHỈ</t>
+  </si>
+  <si>
+    <t>1200001056</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI THANH THANH LIÊM</t>
+  </si>
+  <si>
+    <t>1200001062</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN BOHO CORPORATION</t>
+  </si>
+  <si>
+    <t>1200001065</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ TÂN LÂM</t>
+  </si>
+  <si>
+    <t>1200001072</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH MỘT THÀNH VIÊN KIM CHI</t>
+  </si>
+  <si>
+    <t>1200001077</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SX TM QUANG TRUNG NGUYÊN</t>
+  </si>
+  <si>
+    <t>1200001079</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI - XÂY DỰNG HUY HƯNG</t>
+  </si>
+  <si>
+    <t>1200001084</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SX TM DV SƠN MIỀN TÂY</t>
+  </si>
+  <si>
+    <t>1200001087</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SX-TM SÀI GÒN RIVER VIỆT NAM</t>
+  </si>
+  <si>
+    <t>1200001092</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH HỒNG LUÂN 3</t>
+  </si>
+  <si>
+    <t>1200001094</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH TM SẢN XUẤT XNK NỘI THẤT MCS</t>
+  </si>
+  <si>
+    <t>1200001104</t>
+  </si>
+  <si>
+    <t>CÔNG TY CỔ PHẦN ARTEX ĐỒNG THÁP</t>
+  </si>
+  <si>
+    <t>1200001109</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI DỊCH VỤ XÂY DỰNG THIÊN ĐỊNH</t>
+  </si>
+  <si>
+    <t>1200001113</t>
+  </si>
+  <si>
+    <t>CÔNG TY TRÁCH NHIỆM HỮU HẠN XD SX TM DV AB</t>
+  </si>
+  <si>
+    <t>04</t>
+  </si>
+  <si>
+    <t>1200001114</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI TUÝP NHÔM THUẬN QUÂN</t>
+  </si>
+  <si>
+    <t>1200001118</t>
+  </si>
+  <si>
+    <t>LAZADA</t>
+  </si>
+  <si>
+    <t>1200001119</t>
+  </si>
+  <si>
+    <t>VŨ ĐÌNH DŨNG</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>1200001120</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH TRANSFORMER ROBOTICS PTE</t>
+  </si>
+  <si>
+    <t>1200001123</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SƠN TÀI TRÍ</t>
+  </si>
+  <si>
+    <t>1200001124</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH MTV HOÀNG MINH TUẤN</t>
+  </si>
+  <si>
+    <t>1200001125</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH TRẦN QUÝ</t>
+  </si>
+  <si>
+    <t>1200001144</t>
+  </si>
+  <si>
+    <t>HỘ KINH DOANH BUÔN LÊ COFFEE</t>
+  </si>
+  <si>
+    <t>1200001146</t>
+  </si>
+  <si>
+    <t>TIKTOK</t>
+  </si>
+  <si>
+    <t>06</t>
+  </si>
+  <si>
+    <t>1300000002</t>
+  </si>
+  <si>
+    <t>KODA WOODCRAFT SDN BHD</t>
+  </si>
+  <si>
+    <t>1200000863</t>
+  </si>
+  <si>
+    <t>Công Ty TNHH Thương Mại Tổng Hợp Dũng Lý</t>
+  </si>
+  <si>
+    <t>1200000974</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH CAO VÕ</t>
+  </si>
+  <si>
+    <t>1200001004</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH MỘT THÀNH VIÊN XÂY DỰNG - THƯƠNG MẠI VÀ DỊCH VỤ HOÀNG GIA</t>
+  </si>
+  <si>
+    <t>1200000820</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SẢN XUẤT NỘI THẤT TRẦN TIẾN</t>
+  </si>
+  <si>
+    <t>1200000922</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI XÂY DỰNG TRANG TRÍ NỘI THẤT THỊNH HƯNG</t>
+  </si>
+  <si>
+    <t>1200001148</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH THƯƠNG MẠI DỊCH VỤ THIẾT KẾ AN PHÚ THỊNH</t>
+  </si>
+  <si>
+    <t>1200001027</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH TTK FURNITURE</t>
+  </si>
+  <si>
     <t>1200000888</t>
   </si>
   <si>
     <t>CÔNG TY TNHH ZOE FURNITURE</t>
   </si>
   <si>
-    <t>1200000903</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH CÔNG NGHIỆP NHÀ XANH</t>
-  </si>
-  <si>
-    <t>10811780</t>
-  </si>
-  <si>
-    <t>TẠ DUY HÀ</t>
-  </si>
-  <si>
-    <t>1200000904</t>
-  </si>
-  <si>
-    <t>HỘ KINH DOANH BẢO LÂM</t>
-  </si>
-  <si>
-    <t>1200000935</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN HỆ THỐNG SIÊU THỊ SƠN</t>
-  </si>
-  <si>
-    <t>1200000949</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN BAO BÌ IN KIM LOẠI THẾ KỶ</t>
-  </si>
-  <si>
-    <t>1200000963</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH CƠ KHÍ XÂY DỰNG VIỆT THẮNG</t>
-  </si>
-  <si>
-    <t>1200000971</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ SƠN ANH TÚ</t>
-  </si>
-  <si>
-    <t>1200000973</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH AN THỊNH FURNITURE</t>
-  </si>
-  <si>
-    <t>1200000992</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH DV KT AN TÂM PHÁT</t>
-  </si>
-  <si>
-    <t>1200001011</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN ĐÔNG NGÔ MANUFACTURER</t>
-  </si>
-  <si>
-    <t>1200001023</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI - DỊCH VỤ - XÂY DỰNG MAI TÂM</t>
-  </si>
-  <si>
-    <t>1200001029</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH TRANG TRÍ NỘI THẤT PHONG THẢO</t>
-  </si>
-  <si>
-    <t>10400773</t>
-  </si>
-  <si>
-    <t>VŨ ANH HAI</t>
-  </si>
-  <si>
-    <t>1200001038</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH PHÚ MỸ THĂNG</t>
-  </si>
-  <si>
-    <t>1200001041</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI XÂY DỰNG THIÊN PHÚ DECOR</t>
-  </si>
-  <si>
-    <t>1200001042</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH KIẾN TRÚC GỖ BỌC ĐÔ</t>
-  </si>
-  <si>
-    <t>1200001051</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH VINAWOOD</t>
-  </si>
-  <si>
-    <t>10999776</t>
-  </si>
-  <si>
-    <t>ĐẶNG VĂN CHỈ</t>
-  </si>
-  <si>
-    <t>1200001056</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI THANH THANH LIÊM</t>
-  </si>
-  <si>
-    <t>1200001062</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN BOHO CORPORATION</t>
-  </si>
-  <si>
-    <t>1200001065</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI VÀ DỊCH VỤ TÂN LÂM</t>
-  </si>
-  <si>
-    <t>1200001072</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH MỘT THÀNH VIÊN KIM CHI</t>
-  </si>
-  <si>
-    <t>1200001077</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SX TM QUANG TRUNG NGUYÊN</t>
-  </si>
-  <si>
-    <t>1200001079</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI - XÂY DỰNG HUY HƯNG</t>
-  </si>
-  <si>
-    <t>1200001084</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SX TM DV SƠN MIỀN TÂY</t>
-  </si>
-  <si>
-    <t>1200001087</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SX-TM SÀI GÒN RIVER VIỆT NAM</t>
-  </si>
-  <si>
-    <t>1200001092</t>
-  </si>
-  <si>
-    <t>HỘ KINH DOANH HỒNG LUÂN 3</t>
-  </si>
-  <si>
-    <t>1200001094</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH TM SẢN XUẤT XNK NỘI THẤT MCS</t>
-  </si>
-  <si>
-    <t>1200001104</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN ARTEX ĐỒNG THÁP</t>
-  </si>
-  <si>
-    <t>1200001109</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI DỊCH VỤ XÂY DỰNG THIÊN ĐỊNH</t>
-  </si>
-  <si>
-    <t>1200001113</t>
-  </si>
-  <si>
-    <t>CÔNG TY TRÁCH NHIỆM HỮU HẠN XD SX TM DV AB</t>
-  </si>
-  <si>
-    <t>04</t>
-  </si>
-  <si>
-    <t>1200001114</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SẢN XUẤT THƯƠNG MẠI TUÝP NHÔM THUẬN QUÂN</t>
-  </si>
-  <si>
-    <t>1200001118</t>
-  </si>
-  <si>
-    <t>LAZADA</t>
-  </si>
-  <si>
-    <t>1200001119</t>
-  </si>
-  <si>
-    <t>VŨ ĐÌNH DŨNG</t>
-  </si>
-  <si>
-    <t>0</t>
-  </si>
-  <si>
-    <t>1200001120</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH TRANSFORMER ROBOTICS PTE</t>
-  </si>
-  <si>
-    <t>1200001123</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SƠN TÀI TRÍ</t>
-  </si>
-  <si>
-    <t>1200001124</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH MTV HOÀNG MINH TUẤN</t>
-  </si>
-  <si>
-    <t>1200001125</t>
-  </si>
-  <si>
-    <t>HỘ KINH DOANH TRẦN QUÝ</t>
-  </si>
-  <si>
-    <t>1200001144</t>
-  </si>
-  <si>
-    <t>HỘ KINH DOANH BUÔN LÊ COFFEE</t>
-  </si>
-  <si>
-    <t>06</t>
-  </si>
-  <si>
-    <t>1300000002</t>
-  </si>
-  <si>
-    <t>KODA WOODCRAFT SDN BHD</t>
-  </si>
-  <si>
-    <t>1200000863</t>
-  </si>
-  <si>
-    <t>Công Ty TNHH Thương Mại Tổng Hợp Dũng Lý</t>
-  </si>
-  <si>
-    <t>1200000974</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH CAO VÕ</t>
-  </si>
-  <si>
-    <t>1200001004</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH MỘT THÀNH VIÊN XÂY DỰNG - THƯƠNG MẠI VÀ DỊCH VỤ HOÀNG GIA</t>
-  </si>
-  <si>
-    <t>1200000820</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH SẢN XUẤT NỘI THẤT TRẦN TIẾN</t>
-  </si>
-  <si>
-    <t>1200000922</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI XÂY DỰNG TRANG TRÍ NỘI THẤT THỊNH HƯNG</t>
-  </si>
-  <si>
-    <t>1200000769</t>
-  </si>
-  <si>
-    <t>CÔNG TY CỔ PHẦN KIM MỘC</t>
-  </si>
-  <si>
-    <t>1200000548</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH DAIGAKU (VIỆT NAM)</t>
-  </si>
-  <si>
-    <t>1200001148</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH THƯƠNG MẠI DỊCH VỤ THIẾT KẾ AN PHÚ THỊNH</t>
-  </si>
-  <si>
-    <t>1200001027</t>
-  </si>
-  <si>
-    <t>CÔNG TY TNHH TTK FURNITURE</t>
+    <t>1200000411</t>
+  </si>
+  <si>
+    <t>Công Ty TNHH Chuẩn Tinh - Khanh</t>
+  </si>
+  <si>
+    <t>1200000561</t>
+  </si>
+  <si>
+    <t>CÔNG TY TNHH SX KD XNK NỘI THẤT BOY TẤN</t>
   </si>
   <si>
     <t>Company Code</t>
@@ -1187,7 +1205,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Y100"/>
+  <dimension ref="A1:Y103"/>
   <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="14" bestFit="1" customWidth="1"/>
@@ -1206,9 +1224,11 @@
     <col min="14" max="15" width="12" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="19" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="14" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="11" bestFit="1" customWidth="1"/>
-    <col min="21" max="22" width="15" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="11" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="12" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="11" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="15" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="16" bestFit="1" customWidth="1"/>
     <col min="24" max="24" width="14" bestFit="1" customWidth="1"/>
     <col min="25" max="25" width="19" bestFit="1" customWidth="1"/>
@@ -1216,79 +1236,79 @@
   <sheetData>
     <row r="1" spans="1:25" ht="37.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>249</v>
+        <v>255</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>250</v>
+        <v>256</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="M1" s="3" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="N1" s="3" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="O1" s="3" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="R1" s="3" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="S1" s="3" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="T1" s="3" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="U1" s="3" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="V1" s="3" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="W1" s="3" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="X1" s="3" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" spans="1:25" x14ac:dyDescent="0.25">
@@ -1501,7 +1521,7 @@
         <v>0</v>
       </c>
       <c r="S4" s="2">
-        <v>0</v>
+        <v>103109760</v>
       </c>
       <c r="T4" s="2">
         <v>0</v>
@@ -1519,7 +1539,7 @@
         <v>0</v>
       </c>
       <c r="Y4" s="2">
-        <v>0</v>
+        <v>103109760</v>
       </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.25">
@@ -2040,10 +2060,10 @@
         <v>0</v>
       </c>
       <c r="S11" s="2">
-        <v>0</v>
+        <v>83648270</v>
       </c>
       <c r="T11" s="2">
-        <v>707423134</v>
+        <v>1243745581</v>
       </c>
       <c r="U11" s="2">
         <v>0</v>
@@ -2058,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="Y11" s="2">
-        <v>707423134</v>
+        <v>1327393851</v>
       </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.25">
@@ -3541,10 +3561,10 @@
         <v>4</v>
       </c>
       <c r="F31" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="G31" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="H31" t="s">
         <v>92</v>
@@ -3556,7 +3576,7 @@
         <v>9</v>
       </c>
       <c r="K31" s="2">
-        <v>846730584</v>
+        <v>11043605</v>
       </c>
       <c r="L31" s="2">
         <v>0</v>
@@ -3574,13 +3594,13 @@
         <v>0</v>
       </c>
       <c r="Q31" s="2">
-        <v>846730584</v>
+        <v>11043605</v>
       </c>
       <c r="R31" s="2">
         <v>0</v>
       </c>
       <c r="S31" s="2">
-        <v>0</v>
+        <v>11043605</v>
       </c>
       <c r="T31" s="2">
         <v>0</v>
@@ -3598,7 +3618,7 @@
         <v>0</v>
       </c>
       <c r="Y31" s="2">
-        <v>0</v>
+        <v>11043605</v>
       </c>
     </row>
     <row r="32" spans="1:25" x14ac:dyDescent="0.25">
@@ -3618,10 +3638,10 @@
         <v>4</v>
       </c>
       <c r="F32" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G32" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H32" t="s">
         <v>94</v>
@@ -3633,7 +3653,7 @@
         <v>9</v>
       </c>
       <c r="K32" s="2">
-        <v>1343305728</v>
+        <v>846730584</v>
       </c>
       <c r="L32" s="2">
         <v>0</v>
@@ -3651,7 +3671,7 @@
         <v>0</v>
       </c>
       <c r="Q32" s="2">
-        <v>1343305728</v>
+        <v>846730584</v>
       </c>
       <c r="R32" s="2">
         <v>0</v>
@@ -3695,10 +3715,10 @@
         <v>4</v>
       </c>
       <c r="F33" t="s">
-        <v>10</v>
+        <v>49</v>
       </c>
       <c r="G33" t="s">
-        <v>11</v>
+        <v>50</v>
       </c>
       <c r="H33" t="s">
         <v>96</v>
@@ -3710,13 +3730,13 @@
         <v>9</v>
       </c>
       <c r="K33" s="2">
-        <v>2565161223</v>
+        <v>1343305728</v>
       </c>
       <c r="L33" s="2">
-        <v>3526745660</v>
+        <v>0</v>
       </c>
       <c r="M33" s="2">
-        <v>738941931</v>
+        <v>0</v>
       </c>
       <c r="N33" s="2">
         <v>0</v>
@@ -3728,7 +3748,7 @@
         <v>0</v>
       </c>
       <c r="Q33" s="2">
-        <v>6830848814</v>
+        <v>1343305728</v>
       </c>
       <c r="R33" s="2">
         <v>0</v>
@@ -3772,10 +3792,10 @@
         <v>4</v>
       </c>
       <c r="F34" t="s">
-        <v>49</v>
+        <v>10</v>
       </c>
       <c r="G34" t="s">
-        <v>50</v>
+        <v>11</v>
       </c>
       <c r="H34" t="s">
         <v>98</v>
@@ -3787,13 +3807,13 @@
         <v>9</v>
       </c>
       <c r="K34" s="2">
-        <v>44496000</v>
+        <v>2565161223</v>
       </c>
       <c r="L34" s="2">
-        <v>11607415</v>
+        <v>3526745660</v>
       </c>
       <c r="M34" s="2">
-        <v>0</v>
+        <v>738941931</v>
       </c>
       <c r="N34" s="2">
         <v>0</v>
@@ -3805,7 +3825,7 @@
         <v>0</v>
       </c>
       <c r="Q34" s="2">
-        <v>56103415</v>
+        <v>6830848814</v>
       </c>
       <c r="R34" s="2">
         <v>0</v>
@@ -3814,10 +3834,10 @@
         <v>0</v>
       </c>
       <c r="T34" s="2">
-        <v>0</v>
+        <v>361291643</v>
       </c>
       <c r="U34" s="2">
-        <v>0</v>
+        <v>738941931</v>
       </c>
       <c r="V34" s="2">
         <v>0</v>
@@ -3829,7 +3849,7 @@
         <v>0</v>
       </c>
       <c r="Y34" s="2">
-        <v>0</v>
+        <v>1100233574</v>
       </c>
     </row>
     <row r="35" spans="1:25" x14ac:dyDescent="0.25">
@@ -3849,10 +3869,10 @@
         <v>4</v>
       </c>
       <c r="F35" t="s">
-        <v>19</v>
+        <v>5</v>
       </c>
       <c r="G35" t="s">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="H35" t="s">
         <v>100</v>
@@ -3864,10 +3884,10 @@
         <v>9</v>
       </c>
       <c r="K35" s="2">
-        <v>19077120</v>
+        <v>63436133</v>
       </c>
       <c r="L35" s="2">
-        <v>10790928</v>
+        <v>0</v>
       </c>
       <c r="M35" s="2">
         <v>0</v>
@@ -3882,13 +3902,13 @@
         <v>0</v>
       </c>
       <c r="Q35" s="2">
-        <v>29868048</v>
+        <v>63436133</v>
       </c>
       <c r="R35" s="2">
         <v>0</v>
       </c>
       <c r="S35" s="2">
-        <v>0</v>
+        <v>37748160</v>
       </c>
       <c r="T35" s="2">
         <v>0</v>
@@ -3906,7 +3926,7 @@
         <v>0</v>
       </c>
       <c r="Y35" s="2">
-        <v>0</v>
+        <v>37748160</v>
       </c>
     </row>
     <row r="36" spans="1:25" x14ac:dyDescent="0.25">
@@ -3917,34 +3937,34 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D36" t="s">
         <v>3</v>
       </c>
       <c r="E36" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F36" t="s">
+        <v>49</v>
+      </c>
+      <c r="G36" t="s">
+        <v>50</v>
+      </c>
+      <c r="H36" t="s">
         <v>102</v>
       </c>
-      <c r="G36" t="s">
+      <c r="I36" t="s">
         <v>103</v>
       </c>
-      <c r="H36" t="s">
-        <v>104</v>
-      </c>
-      <c r="I36" t="s">
-        <v>105</v>
-      </c>
       <c r="J36" t="s">
         <v>9</v>
       </c>
       <c r="K36" s="2">
-        <v>68591463</v>
+        <v>44496000</v>
       </c>
       <c r="L36" s="2">
-        <v>0</v>
+        <v>11607415</v>
       </c>
       <c r="M36" s="2">
         <v>0</v>
@@ -3959,7 +3979,7 @@
         <v>0</v>
       </c>
       <c r="Q36" s="2">
-        <v>68591463</v>
+        <v>56103415</v>
       </c>
       <c r="R36" s="2">
         <v>0</v>
@@ -3994,34 +4014,34 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D37" t="s">
         <v>3</v>
       </c>
       <c r="E37" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="F37" t="s">
-        <v>107</v>
+        <v>19</v>
       </c>
       <c r="G37" t="s">
-        <v>108</v>
+        <v>20</v>
       </c>
       <c r="H37" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="I37" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="J37" t="s">
         <v>9</v>
       </c>
       <c r="K37" s="2">
-        <v>23259938</v>
+        <v>19077120</v>
       </c>
       <c r="L37" s="2">
-        <v>9321398</v>
+        <v>10790928</v>
       </c>
       <c r="M37" s="2">
         <v>0</v>
@@ -4036,7 +4056,7 @@
         <v>0</v>
       </c>
       <c r="Q37" s="2">
-        <v>32581336</v>
+        <v>29868048</v>
       </c>
       <c r="R37" s="2">
         <v>0</v>
@@ -4080,22 +4100,22 @@
         <v>80</v>
       </c>
       <c r="F38" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="G38" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="H38" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="I38" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="J38" t="s">
         <v>9</v>
       </c>
       <c r="K38" s="2">
-        <v>68546328</v>
+        <v>68591463</v>
       </c>
       <c r="L38" s="2">
         <v>0</v>
@@ -4113,13 +4133,13 @@
         <v>0</v>
       </c>
       <c r="Q38" s="2">
-        <v>68546328</v>
+        <v>68591463</v>
       </c>
       <c r="R38" s="2">
         <v>0</v>
       </c>
       <c r="S38" s="2">
-        <v>23886291</v>
+        <v>48246984</v>
       </c>
       <c r="T38" s="2">
         <v>0</v>
@@ -4137,7 +4157,7 @@
         <v>0</v>
       </c>
       <c r="Y38" s="2">
-        <v>23886291</v>
+        <v>48246984</v>
       </c>
     </row>
     <row r="39" spans="1:25" x14ac:dyDescent="0.25">
@@ -4154,7 +4174,7 @@
         <v>3</v>
       </c>
       <c r="E39" t="s">
-        <v>80</v>
+        <v>110</v>
       </c>
       <c r="F39" t="s">
         <v>111</v>
@@ -4163,19 +4183,19 @@
         <v>112</v>
       </c>
       <c r="H39" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="I39" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="J39" t="s">
         <v>9</v>
       </c>
       <c r="K39" s="2">
-        <v>587755726</v>
+        <v>23259938</v>
       </c>
       <c r="L39" s="2">
-        <v>424340449</v>
+        <v>9321398</v>
       </c>
       <c r="M39" s="2">
         <v>0</v>
@@ -4190,16 +4210,16 @@
         <v>0</v>
       </c>
       <c r="Q39" s="2">
-        <v>1012096175</v>
+        <v>32581336</v>
       </c>
       <c r="R39" s="2">
         <v>0</v>
       </c>
       <c r="S39" s="2">
-        <v>0</v>
+        <v>15786891</v>
       </c>
       <c r="T39" s="2">
-        <v>200000000</v>
+        <v>0</v>
       </c>
       <c r="U39" s="2">
         <v>0</v>
@@ -4214,7 +4234,7 @@
         <v>0</v>
       </c>
       <c r="Y39" s="2">
-        <v>200000000</v>
+        <v>15786891</v>
       </c>
     </row>
     <row r="40" spans="1:25" x14ac:dyDescent="0.25">
@@ -4234,10 +4254,10 @@
         <v>80</v>
       </c>
       <c r="F40" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="G40" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="H40" t="s">
         <v>117</v>
@@ -4249,7 +4269,7 @@
         <v>9</v>
       </c>
       <c r="K40" s="2">
-        <v>305651559</v>
+        <v>68546328</v>
       </c>
       <c r="L40" s="2">
         <v>0</v>
@@ -4267,13 +4287,13 @@
         <v>0</v>
       </c>
       <c r="Q40" s="2">
-        <v>305651559</v>
+        <v>68546328</v>
       </c>
       <c r="R40" s="2">
         <v>0</v>
       </c>
       <c r="S40" s="2">
-        <v>48581001</v>
+        <v>23886291</v>
       </c>
       <c r="T40" s="2">
         <v>0</v>
@@ -4291,7 +4311,7 @@
         <v>0</v>
       </c>
       <c r="Y40" s="2">
-        <v>48581001</v>
+        <v>23886291</v>
       </c>
     </row>
     <row r="41" spans="1:25" x14ac:dyDescent="0.25">
@@ -4308,34 +4328,34 @@
         <v>3</v>
       </c>
       <c r="E41" t="s">
+        <v>80</v>
+      </c>
+      <c r="F41" t="s">
+        <v>115</v>
+      </c>
+      <c r="G41" t="s">
+        <v>116</v>
+      </c>
+      <c r="H41" t="s">
         <v>119</v>
       </c>
-      <c r="F41" t="s">
-        <v>107</v>
-      </c>
-      <c r="G41" t="s">
-        <v>108</v>
-      </c>
-      <c r="H41" t="s">
+      <c r="I41" t="s">
         <v>120</v>
       </c>
-      <c r="I41" t="s">
-        <v>121</v>
-      </c>
       <c r="J41" t="s">
         <v>9</v>
       </c>
       <c r="K41" s="2">
-        <v>0</v>
+        <v>587755726</v>
       </c>
       <c r="L41" s="2">
-        <v>0</v>
+        <v>424340449</v>
       </c>
       <c r="M41" s="2">
         <v>0</v>
       </c>
       <c r="N41" s="2">
-        <v>36336913</v>
+        <v>0</v>
       </c>
       <c r="O41" s="2">
         <v>0</v>
@@ -4344,7 +4364,7 @@
         <v>0</v>
       </c>
       <c r="Q41" s="2">
-        <v>36336913</v>
+        <v>1012096175</v>
       </c>
       <c r="R41" s="2">
         <v>0</v>
@@ -4353,7 +4373,7 @@
         <v>0</v>
       </c>
       <c r="T41" s="2">
-        <v>0</v>
+        <v>200000000</v>
       </c>
       <c r="U41" s="2">
         <v>0</v>
@@ -4368,7 +4388,7 @@
         <v>0</v>
       </c>
       <c r="Y41" s="2">
-        <v>0</v>
+        <v>200000000</v>
       </c>
     </row>
     <row r="42" spans="1:25" x14ac:dyDescent="0.25">
@@ -4388,22 +4408,22 @@
         <v>80</v>
       </c>
       <c r="F42" t="s">
+        <v>106</v>
+      </c>
+      <c r="G42" t="s">
         <v>107</v>
       </c>
-      <c r="G42" t="s">
-        <v>108</v>
-      </c>
       <c r="H42" t="s">
+        <v>121</v>
+      </c>
+      <c r="I42" t="s">
         <v>122</v>
       </c>
-      <c r="I42" t="s">
-        <v>123</v>
-      </c>
       <c r="J42" t="s">
         <v>9</v>
       </c>
       <c r="K42" s="2">
-        <v>430866875</v>
+        <v>305651559</v>
       </c>
       <c r="L42" s="2">
         <v>0</v>
@@ -4421,13 +4441,13 @@
         <v>0</v>
       </c>
       <c r="Q42" s="2">
-        <v>430866875</v>
+        <v>305651559</v>
       </c>
       <c r="R42" s="2">
         <v>0</v>
       </c>
       <c r="S42" s="2">
-        <v>144789230</v>
+        <v>48581001</v>
       </c>
       <c r="T42" s="2">
         <v>0</v>
@@ -4445,7 +4465,7 @@
         <v>0</v>
       </c>
       <c r="Y42" s="2">
-        <v>144789230</v>
+        <v>48581001</v>
       </c>
     </row>
     <row r="43" spans="1:25" x14ac:dyDescent="0.25">
@@ -4462,13 +4482,13 @@
         <v>3</v>
       </c>
       <c r="E43" t="s">
-        <v>80</v>
+        <v>123</v>
       </c>
       <c r="F43" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="G43" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="H43" t="s">
         <v>124</v>
@@ -4480,7 +4500,7 @@
         <v>9</v>
       </c>
       <c r="K43" s="2">
-        <v>316905738</v>
+        <v>0</v>
       </c>
       <c r="L43" s="2">
         <v>0</v>
@@ -4489,7 +4509,7 @@
         <v>0</v>
       </c>
       <c r="N43" s="2">
-        <v>0</v>
+        <v>36336913</v>
       </c>
       <c r="O43" s="2">
         <v>0</v>
@@ -4498,7 +4518,7 @@
         <v>0</v>
       </c>
       <c r="Q43" s="2">
-        <v>316905738</v>
+        <v>36336913</v>
       </c>
       <c r="R43" s="2">
         <v>0</v>
@@ -4539,25 +4559,25 @@
         <v>3</v>
       </c>
       <c r="E44" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="F44" t="s">
+        <v>111</v>
+      </c>
+      <c r="G44" t="s">
+        <v>112</v>
+      </c>
+      <c r="H44" t="s">
         <v>126</v>
       </c>
-      <c r="G44" t="s">
+      <c r="I44" t="s">
         <v>127</v>
       </c>
-      <c r="H44" t="s">
-        <v>128</v>
-      </c>
-      <c r="I44" t="s">
-        <v>129</v>
-      </c>
       <c r="J44" t="s">
         <v>9</v>
       </c>
       <c r="K44" s="2">
-        <v>12185731</v>
+        <v>430866875</v>
       </c>
       <c r="L44" s="2">
         <v>0</v>
@@ -4569,19 +4589,19 @@
         <v>0</v>
       </c>
       <c r="O44" s="2">
-        <v>-437763</v>
+        <v>0</v>
       </c>
       <c r="P44" s="2">
-        <v>-563094</v>
+        <v>0</v>
       </c>
       <c r="Q44" s="2">
-        <v>11184874</v>
+        <v>430866875</v>
       </c>
       <c r="R44" s="2">
         <v>0</v>
       </c>
       <c r="S44" s="2">
-        <v>0</v>
+        <v>144789230</v>
       </c>
       <c r="T44" s="2">
         <v>0</v>
@@ -4599,7 +4619,7 @@
         <v>0</v>
       </c>
       <c r="Y44" s="2">
-        <v>0</v>
+        <v>144789230</v>
       </c>
     </row>
     <row r="45" spans="1:25" x14ac:dyDescent="0.25">
@@ -4616,25 +4636,25 @@
         <v>3</v>
       </c>
       <c r="E45" t="s">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="F45" t="s">
-        <v>126</v>
+        <v>111</v>
       </c>
       <c r="G45" t="s">
-        <v>127</v>
+        <v>112</v>
       </c>
       <c r="H45" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="I45" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J45" t="s">
         <v>9</v>
       </c>
       <c r="K45" s="2">
-        <v>6064313</v>
+        <v>316905738</v>
       </c>
       <c r="L45" s="2">
         <v>0</v>
@@ -4649,10 +4669,10 @@
         <v>0</v>
       </c>
       <c r="P45" s="2">
-        <v>-731234</v>
+        <v>0</v>
       </c>
       <c r="Q45" s="2">
-        <v>5333079</v>
+        <v>316905738</v>
       </c>
       <c r="R45" s="2">
         <v>0</v>
@@ -4693,13 +4713,13 @@
         <v>3</v>
       </c>
       <c r="E46" t="s">
-        <v>80</v>
+        <v>123</v>
       </c>
       <c r="F46" t="s">
-        <v>81</v>
+        <v>130</v>
       </c>
       <c r="G46" t="s">
-        <v>82</v>
+        <v>131</v>
       </c>
       <c r="H46" t="s">
         <v>132</v>
@@ -4711,10 +4731,10 @@
         <v>9</v>
       </c>
       <c r="K46" s="2">
-        <v>3404957</v>
+        <v>12185731</v>
       </c>
       <c r="L46" s="2">
-        <v>-286417</v>
+        <v>0</v>
       </c>
       <c r="M46" s="2">
         <v>0</v>
@@ -4723,13 +4743,13 @@
         <v>0</v>
       </c>
       <c r="O46" s="2">
-        <v>0</v>
+        <v>-437763</v>
       </c>
       <c r="P46" s="2">
-        <v>0</v>
+        <v>-563094</v>
       </c>
       <c r="Q46" s="2">
-        <v>3118540</v>
+        <v>11184874</v>
       </c>
       <c r="R46" s="2">
         <v>0</v>
@@ -4770,13 +4790,13 @@
         <v>3</v>
       </c>
       <c r="E47" t="s">
-        <v>119</v>
+        <v>110</v>
       </c>
       <c r="F47" t="s">
-        <v>102</v>
+        <v>130</v>
       </c>
       <c r="G47" t="s">
-        <v>103</v>
+        <v>131</v>
       </c>
       <c r="H47" t="s">
         <v>134</v>
@@ -4788,7 +4808,7 @@
         <v>9</v>
       </c>
       <c r="K47" s="2">
-        <v>0</v>
+        <v>6064313</v>
       </c>
       <c r="L47" s="2">
         <v>0</v>
@@ -4803,10 +4823,10 @@
         <v>0</v>
       </c>
       <c r="P47" s="2">
-        <v>18628426</v>
+        <v>-731234</v>
       </c>
       <c r="Q47" s="2">
-        <v>18628426</v>
+        <v>5333079</v>
       </c>
       <c r="R47" s="2">
         <v>0</v>
@@ -4847,7 +4867,7 @@
         <v>3</v>
       </c>
       <c r="E48" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="F48" t="s">
         <v>81</v>
@@ -4865,10 +4885,10 @@
         <v>9</v>
       </c>
       <c r="K48" s="2">
-        <v>54441960</v>
+        <v>3404957</v>
       </c>
       <c r="L48" s="2">
-        <v>0</v>
+        <v>-286417</v>
       </c>
       <c r="M48" s="2">
         <v>0</v>
@@ -4883,7 +4903,7 @@
         <v>0</v>
       </c>
       <c r="Q48" s="2">
-        <v>54441960</v>
+        <v>3118540</v>
       </c>
       <c r="R48" s="2">
         <v>0</v>
@@ -4924,13 +4944,13 @@
         <v>3</v>
       </c>
       <c r="E49" t="s">
-        <v>80</v>
+        <v>123</v>
       </c>
       <c r="F49" t="s">
-        <v>81</v>
+        <v>106</v>
       </c>
       <c r="G49" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="H49" t="s">
         <v>138</v>
@@ -4945,22 +4965,22 @@
         <v>0</v>
       </c>
       <c r="L49" s="2">
-        <v>8553717</v>
+        <v>0</v>
       </c>
       <c r="M49" s="2">
-        <v>38598624</v>
+        <v>0</v>
       </c>
       <c r="N49" s="2">
         <v>0</v>
       </c>
       <c r="O49" s="2">
-        <v>47819368</v>
+        <v>0</v>
       </c>
       <c r="P49" s="2">
-        <v>0</v>
+        <v>18628426</v>
       </c>
       <c r="Q49" s="2">
-        <v>94971709</v>
+        <v>18628426</v>
       </c>
       <c r="R49" s="2">
         <v>0</v>
@@ -4995,31 +5015,31 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D50" t="s">
         <v>3</v>
       </c>
       <c r="E50" t="s">
+        <v>123</v>
+      </c>
+      <c r="F50" t="s">
+        <v>81</v>
+      </c>
+      <c r="G50" t="s">
+        <v>82</v>
+      </c>
+      <c r="H50" t="s">
         <v>140</v>
       </c>
-      <c r="F50" t="s">
-        <v>65</v>
-      </c>
-      <c r="G50" t="s">
-        <v>66</v>
-      </c>
-      <c r="H50" t="s">
+      <c r="I50" t="s">
         <v>141</v>
       </c>
-      <c r="I50" t="s">
-        <v>142</v>
-      </c>
       <c r="J50" t="s">
         <v>9</v>
       </c>
       <c r="K50" s="2">
-        <v>38394000</v>
+        <v>54441960</v>
       </c>
       <c r="L50" s="2">
         <v>0</v>
@@ -5037,7 +5057,7 @@
         <v>0</v>
       </c>
       <c r="Q50" s="2">
-        <v>38394000</v>
+        <v>54441960</v>
       </c>
       <c r="R50" s="2">
         <v>0</v>
@@ -5072,49 +5092,49 @@
         <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="D51" t="s">
         <v>3</v>
       </c>
       <c r="E51" t="s">
-        <v>140</v>
+        <v>80</v>
       </c>
       <c r="F51" t="s">
-        <v>65</v>
+        <v>81</v>
       </c>
       <c r="G51" t="s">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="H51" t="s">
+        <v>142</v>
+      </c>
+      <c r="I51" t="s">
         <v>143</v>
       </c>
-      <c r="I51" t="s">
-        <v>144</v>
-      </c>
       <c r="J51" t="s">
         <v>9</v>
       </c>
       <c r="K51" s="2">
-        <v>107244000</v>
+        <v>0</v>
       </c>
       <c r="L51" s="2">
-        <v>14874800</v>
+        <v>8553717</v>
       </c>
       <c r="M51" s="2">
-        <v>0</v>
+        <v>38598624</v>
       </c>
       <c r="N51" s="2">
         <v>0</v>
       </c>
       <c r="O51" s="2">
-        <v>0</v>
+        <v>47819368</v>
       </c>
       <c r="P51" s="2">
         <v>0</v>
       </c>
       <c r="Q51" s="2">
-        <v>122118800</v>
+        <v>94971709</v>
       </c>
       <c r="R51" s="2">
         <v>0</v>
@@ -5149,19 +5169,19 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="D52" t="s">
         <v>3</v>
       </c>
       <c r="E52" t="s">
-        <v>4</v>
+        <v>144</v>
       </c>
       <c r="F52" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="G52" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="H52" t="s">
         <v>145</v>
@@ -5173,7 +5193,7 @@
         <v>9</v>
       </c>
       <c r="K52" s="2">
-        <v>15683328</v>
+        <v>38394000</v>
       </c>
       <c r="L52" s="2">
         <v>0</v>
@@ -5191,7 +5211,7 @@
         <v>0</v>
       </c>
       <c r="Q52" s="2">
-        <v>15683328</v>
+        <v>38394000</v>
       </c>
       <c r="R52" s="2">
         <v>0</v>
@@ -5226,19 +5246,19 @@
         <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="D53" t="s">
         <v>3</v>
       </c>
       <c r="E53" t="s">
-        <v>4</v>
+        <v>144</v>
       </c>
       <c r="F53" t="s">
-        <v>19</v>
+        <v>65</v>
       </c>
       <c r="G53" t="s">
-        <v>20</v>
+        <v>66</v>
       </c>
       <c r="H53" t="s">
         <v>147</v>
@@ -5250,10 +5270,10 @@
         <v>9</v>
       </c>
       <c r="K53" s="2">
-        <v>234264960</v>
+        <v>107244000</v>
       </c>
       <c r="L53" s="2">
-        <v>81294624</v>
+        <v>14874800</v>
       </c>
       <c r="M53" s="2">
         <v>0</v>
@@ -5268,7 +5288,7 @@
         <v>0</v>
       </c>
       <c r="Q53" s="2">
-        <v>315559584</v>
+        <v>122118800</v>
       </c>
       <c r="R53" s="2">
         <v>0</v>
@@ -5303,34 +5323,34 @@
         <v>1</v>
       </c>
       <c r="C54" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D54" t="s">
         <v>3</v>
       </c>
       <c r="E54" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F54" t="s">
+        <v>19</v>
+      </c>
+      <c r="G54" t="s">
+        <v>20</v>
+      </c>
+      <c r="H54" t="s">
         <v>149</v>
       </c>
-      <c r="G54" t="s">
+      <c r="I54" t="s">
         <v>150</v>
       </c>
-      <c r="H54" t="s">
-        <v>151</v>
-      </c>
-      <c r="I54" t="s">
-        <v>152</v>
-      </c>
       <c r="J54" t="s">
         <v>9</v>
       </c>
       <c r="K54" s="2">
-        <v>44298144</v>
+        <v>234264960</v>
       </c>
       <c r="L54" s="2">
-        <v>0</v>
+        <v>81294624</v>
       </c>
       <c r="M54" s="2">
         <v>0</v>
@@ -5345,7 +5365,7 @@
         <v>0</v>
       </c>
       <c r="Q54" s="2">
-        <v>44298144</v>
+        <v>315559584</v>
       </c>
       <c r="R54" s="2">
         <v>0</v>
@@ -5386,13 +5406,13 @@
         <v>3</v>
       </c>
       <c r="E55" t="s">
-        <v>106</v>
+        <v>80</v>
       </c>
       <c r="F55" t="s">
-        <v>102</v>
+        <v>151</v>
       </c>
       <c r="G55" t="s">
-        <v>103</v>
+        <v>152</v>
       </c>
       <c r="H55" t="s">
         <v>153</v>
@@ -5404,10 +5424,10 @@
         <v>9</v>
       </c>
       <c r="K55" s="2">
-        <v>0</v>
+        <v>44298144</v>
       </c>
       <c r="L55" s="2">
-        <v>21506679</v>
+        <v>0</v>
       </c>
       <c r="M55" s="2">
         <v>0</v>
@@ -5422,7 +5442,7 @@
         <v>0</v>
       </c>
       <c r="Q55" s="2">
-        <v>21506679</v>
+        <v>44298144</v>
       </c>
       <c r="R55" s="2">
         <v>0</v>
@@ -5457,19 +5477,19 @@
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D56" t="s">
         <v>3</v>
       </c>
       <c r="E56" t="s">
-        <v>4</v>
+        <v>110</v>
       </c>
       <c r="F56" t="s">
-        <v>43</v>
+        <v>106</v>
       </c>
       <c r="G56" t="s">
-        <v>44</v>
+        <v>107</v>
       </c>
       <c r="H56" t="s">
         <v>155</v>
@@ -5481,10 +5501,10 @@
         <v>9</v>
       </c>
       <c r="K56" s="2">
-        <v>201139200</v>
+        <v>0</v>
       </c>
       <c r="L56" s="2">
-        <v>0</v>
+        <v>21506679</v>
       </c>
       <c r="M56" s="2">
         <v>0</v>
@@ -5499,7 +5519,7 @@
         <v>0</v>
       </c>
       <c r="Q56" s="2">
-        <v>201139200</v>
+        <v>21506679</v>
       </c>
       <c r="R56" s="2">
         <v>0</v>
@@ -5543,10 +5563,10 @@
         <v>4</v>
       </c>
       <c r="F57" t="s">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="G57" t="s">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="H57" t="s">
         <v>157</v>
@@ -5558,7 +5578,7 @@
         <v>9</v>
       </c>
       <c r="K57" s="2">
-        <v>2565648</v>
+        <v>201139200</v>
       </c>
       <c r="L57" s="2">
         <v>0</v>
@@ -5576,7 +5596,7 @@
         <v>0</v>
       </c>
       <c r="Q57" s="2">
-        <v>2565648</v>
+        <v>201139200</v>
       </c>
       <c r="R57" s="2">
         <v>0</v>
@@ -5611,19 +5631,19 @@
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D58" t="s">
         <v>3</v>
       </c>
       <c r="E58" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F58" t="s">
-        <v>111</v>
+        <v>5</v>
       </c>
       <c r="G58" t="s">
-        <v>112</v>
+        <v>6</v>
       </c>
       <c r="H58" t="s">
         <v>159</v>
@@ -5635,7 +5655,7 @@
         <v>9</v>
       </c>
       <c r="K58" s="2">
-        <v>93045016</v>
+        <v>2565648</v>
       </c>
       <c r="L58" s="2">
         <v>0</v>
@@ -5653,7 +5673,7 @@
         <v>0</v>
       </c>
       <c r="Q58" s="2">
-        <v>93045016</v>
+        <v>2565648</v>
       </c>
       <c r="R58" s="2">
         <v>0</v>
@@ -5688,19 +5708,19 @@
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D59" t="s">
         <v>3</v>
       </c>
       <c r="E59" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F59" t="s">
-        <v>5</v>
+        <v>115</v>
       </c>
       <c r="G59" t="s">
-        <v>6</v>
+        <v>116</v>
       </c>
       <c r="H59" t="s">
         <v>161</v>
@@ -5712,7 +5732,7 @@
         <v>9</v>
       </c>
       <c r="K59" s="2">
-        <v>5769792</v>
+        <v>93045016</v>
       </c>
       <c r="L59" s="2">
         <v>0</v>
@@ -5730,7 +5750,7 @@
         <v>0</v>
       </c>
       <c r="Q59" s="2">
-        <v>5769792</v>
+        <v>93045016</v>
       </c>
       <c r="R59" s="2">
         <v>0</v>
@@ -5765,19 +5785,19 @@
         <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>63</v>
+        <v>2</v>
       </c>
       <c r="D60" t="s">
         <v>3</v>
       </c>
       <c r="E60" t="s">
-        <v>140</v>
+        <v>4</v>
       </c>
       <c r="F60" t="s">
-        <v>65</v>
+        <v>5</v>
       </c>
       <c r="G60" t="s">
-        <v>66</v>
+        <v>6</v>
       </c>
       <c r="H60" t="s">
         <v>163</v>
@@ -5789,7 +5809,7 @@
         <v>9</v>
       </c>
       <c r="K60" s="2">
-        <v>3631392</v>
+        <v>5769792</v>
       </c>
       <c r="L60" s="2">
         <v>0</v>
@@ -5807,7 +5827,7 @@
         <v>0</v>
       </c>
       <c r="Q60" s="2">
-        <v>3631392</v>
+        <v>5769792</v>
       </c>
       <c r="R60" s="2">
         <v>0</v>
@@ -5842,19 +5862,19 @@
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>2</v>
+        <v>63</v>
       </c>
       <c r="D61" t="s">
         <v>3</v>
       </c>
       <c r="E61" t="s">
-        <v>4</v>
+        <v>144</v>
       </c>
       <c r="F61" t="s">
-        <v>49</v>
+        <v>65</v>
       </c>
       <c r="G61" t="s">
-        <v>50</v>
+        <v>66</v>
       </c>
       <c r="H61" t="s">
         <v>165</v>
@@ -5866,7 +5886,7 @@
         <v>9</v>
       </c>
       <c r="K61" s="2">
-        <v>303350184</v>
+        <v>3631392</v>
       </c>
       <c r="L61" s="2">
         <v>0</v>
@@ -5884,7 +5904,7 @@
         <v>0</v>
       </c>
       <c r="Q61" s="2">
-        <v>303350184</v>
+        <v>3631392</v>
       </c>
       <c r="R61" s="2">
         <v>0</v>
@@ -5919,19 +5939,19 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D62" t="s">
         <v>3</v>
       </c>
       <c r="E62" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="F62" t="s">
-        <v>102</v>
+        <v>49</v>
       </c>
       <c r="G62" t="s">
-        <v>103</v>
+        <v>50</v>
       </c>
       <c r="H62" t="s">
         <v>167</v>
@@ -5943,7 +5963,7 @@
         <v>9</v>
       </c>
       <c r="K62" s="2">
-        <v>11767702</v>
+        <v>303350184</v>
       </c>
       <c r="L62" s="2">
         <v>0</v>
@@ -5961,7 +5981,7 @@
         <v>0</v>
       </c>
       <c r="Q62" s="2">
-        <v>11767702</v>
+        <v>303350184</v>
       </c>
       <c r="R62" s="2">
         <v>0</v>
@@ -6002,13 +6022,13 @@
         <v>3</v>
       </c>
       <c r="E63" t="s">
+        <v>110</v>
+      </c>
+      <c r="F63" t="s">
         <v>106</v>
       </c>
-      <c r="F63" t="s">
-        <v>81</v>
-      </c>
       <c r="G63" t="s">
-        <v>82</v>
+        <v>107</v>
       </c>
       <c r="H63" t="s">
         <v>169</v>
@@ -6020,7 +6040,7 @@
         <v>9</v>
       </c>
       <c r="K63" s="2">
-        <v>0</v>
+        <v>11767702</v>
       </c>
       <c r="L63" s="2">
         <v>0</v>
@@ -6035,10 +6055,10 @@
         <v>0</v>
       </c>
       <c r="P63" s="2">
-        <v>30207046</v>
+        <v>0</v>
       </c>
       <c r="Q63" s="2">
-        <v>30207046</v>
+        <v>11767702</v>
       </c>
       <c r="R63" s="2">
         <v>0</v>
@@ -6079,20 +6099,20 @@
         <v>3</v>
       </c>
       <c r="E64" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F64" t="s">
+        <v>81</v>
+      </c>
+      <c r="G64" t="s">
+        <v>82</v>
+      </c>
+      <c r="H64" t="s">
         <v>171</v>
       </c>
-      <c r="G64" t="s">
+      <c r="I64" t="s">
         <v>172</v>
       </c>
-      <c r="H64" t="s">
-        <v>169</v>
-      </c>
-      <c r="I64" t="s">
-        <v>170</v>
-      </c>
       <c r="J64" t="s">
         <v>9</v>
       </c>
@@ -6112,10 +6132,10 @@
         <v>0</v>
       </c>
       <c r="P64" s="2">
-        <v>8518911</v>
+        <v>30207046</v>
       </c>
       <c r="Q64" s="2">
-        <v>8518911</v>
+        <v>30207046</v>
       </c>
       <c r="R64" s="2">
         <v>0</v>
@@ -6150,31 +6170,31 @@
         <v>1</v>
       </c>
       <c r="C65" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D65" t="s">
         <v>3</v>
       </c>
       <c r="E65" t="s">
-        <v>4</v>
+        <v>110</v>
       </c>
       <c r="F65" t="s">
-        <v>5</v>
+        <v>173</v>
       </c>
       <c r="G65" t="s">
-        <v>6</v>
+        <v>174</v>
       </c>
       <c r="H65" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I65" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="J65" t="s">
         <v>9</v>
       </c>
       <c r="K65" s="2">
-        <v>172499760</v>
+        <v>0</v>
       </c>
       <c r="L65" s="2">
         <v>0</v>
@@ -6189,10 +6209,10 @@
         <v>0</v>
       </c>
       <c r="P65" s="2">
-        <v>0</v>
+        <v>8518911</v>
       </c>
       <c r="Q65" s="2">
-        <v>172499760</v>
+        <v>8518911</v>
       </c>
       <c r="R65" s="2">
         <v>0</v>
@@ -6227,19 +6247,19 @@
         <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D66" t="s">
         <v>3</v>
       </c>
       <c r="E66" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F66" t="s">
-        <v>102</v>
+        <v>5</v>
       </c>
       <c r="G66" t="s">
-        <v>103</v>
+        <v>6</v>
       </c>
       <c r="H66" t="s">
         <v>175</v>
@@ -6251,7 +6271,7 @@
         <v>9</v>
       </c>
       <c r="K66" s="2">
-        <v>14786158</v>
+        <v>172499760</v>
       </c>
       <c r="L66" s="2">
         <v>0</v>
@@ -6269,7 +6289,7 @@
         <v>0</v>
       </c>
       <c r="Q66" s="2">
-        <v>14786158</v>
+        <v>172499760</v>
       </c>
       <c r="R66" s="2">
         <v>0</v>
@@ -6304,19 +6324,19 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D67" t="s">
         <v>3</v>
       </c>
       <c r="E67" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F67" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="G67" t="s">
-        <v>16</v>
+        <v>107</v>
       </c>
       <c r="H67" t="s">
         <v>177</v>
@@ -6328,7 +6348,7 @@
         <v>9</v>
       </c>
       <c r="K67" s="2">
-        <v>48819936</v>
+        <v>14786158</v>
       </c>
       <c r="L67" s="2">
         <v>0</v>
@@ -6346,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="Q67" s="2">
-        <v>48819936</v>
+        <v>14786158</v>
       </c>
       <c r="R67" s="2">
         <v>0</v>
@@ -6390,10 +6410,10 @@
         <v>4</v>
       </c>
       <c r="F68" t="s">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="G68" t="s">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="H68" t="s">
         <v>179</v>
@@ -6405,10 +6425,10 @@
         <v>9</v>
       </c>
       <c r="K68" s="2">
-        <v>49120000</v>
+        <v>48819936</v>
       </c>
       <c r="L68" s="2">
-        <v>245569000</v>
+        <v>0</v>
       </c>
       <c r="M68" s="2">
         <v>0</v>
@@ -6423,7 +6443,7 @@
         <v>0</v>
       </c>
       <c r="Q68" s="2">
-        <v>294689000</v>
+        <v>48819936</v>
       </c>
       <c r="R68" s="2">
         <v>0</v>
@@ -6467,25 +6487,25 @@
         <v>4</v>
       </c>
       <c r="F69" t="s">
+        <v>19</v>
+      </c>
+      <c r="G69" t="s">
+        <v>20</v>
+      </c>
+      <c r="H69" t="s">
         <v>181</v>
       </c>
-      <c r="G69" t="s">
+      <c r="I69" t="s">
         <v>182</v>
       </c>
-      <c r="H69" t="s">
-        <v>183</v>
-      </c>
-      <c r="I69" t="s">
-        <v>184</v>
-      </c>
       <c r="J69" t="s">
         <v>9</v>
       </c>
       <c r="K69" s="2">
-        <v>28691280</v>
+        <v>49120000</v>
       </c>
       <c r="L69" s="2">
-        <v>35977392</v>
+        <v>245569000</v>
       </c>
       <c r="M69" s="2">
         <v>0</v>
@@ -6500,7 +6520,7 @@
         <v>0</v>
       </c>
       <c r="Q69" s="2">
-        <v>64668672</v>
+        <v>294689000</v>
       </c>
       <c r="R69" s="2">
         <v>0</v>
@@ -6544,10 +6564,10 @@
         <v>4</v>
       </c>
       <c r="F70" t="s">
-        <v>49</v>
+        <v>183</v>
       </c>
       <c r="G70" t="s">
-        <v>50</v>
+        <v>184</v>
       </c>
       <c r="H70" t="s">
         <v>185</v>
@@ -6559,10 +6579,10 @@
         <v>9</v>
       </c>
       <c r="K70" s="2">
-        <v>555141168</v>
+        <v>28691280</v>
       </c>
       <c r="L70" s="2">
-        <v>0</v>
+        <v>35977392</v>
       </c>
       <c r="M70" s="2">
         <v>0</v>
@@ -6577,7 +6597,7 @@
         <v>0</v>
       </c>
       <c r="Q70" s="2">
-        <v>555141168</v>
+        <v>64668672</v>
       </c>
       <c r="R70" s="2">
         <v>0</v>
@@ -6612,19 +6632,19 @@
         <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D71" t="s">
         <v>3</v>
       </c>
       <c r="E71" t="s">
-        <v>106</v>
+        <v>4</v>
       </c>
       <c r="F71" t="s">
-        <v>107</v>
+        <v>49</v>
       </c>
       <c r="G71" t="s">
-        <v>108</v>
+        <v>50</v>
       </c>
       <c r="H71" t="s">
         <v>187</v>
@@ -6636,31 +6656,31 @@
         <v>9</v>
       </c>
       <c r="K71" s="2">
-        <v>15037055</v>
+        <v>555141168</v>
       </c>
       <c r="L71" s="2">
-        <v>10235715</v>
+        <v>0</v>
       </c>
       <c r="M71" s="2">
-        <v>8519043</v>
+        <v>0</v>
       </c>
       <c r="N71" s="2">
         <v>0</v>
       </c>
       <c r="O71" s="2">
-        <v>29470499</v>
+        <v>0</v>
       </c>
       <c r="P71" s="2">
         <v>0</v>
       </c>
       <c r="Q71" s="2">
-        <v>63262312</v>
+        <v>555141168</v>
       </c>
       <c r="R71" s="2">
         <v>0</v>
       </c>
       <c r="S71" s="2">
-        <v>0</v>
+        <v>127590768</v>
       </c>
       <c r="T71" s="2">
         <v>0</v>
@@ -6678,7 +6698,7 @@
         <v>0</v>
       </c>
       <c r="Y71" s="2">
-        <v>0</v>
+        <v>127590768</v>
       </c>
     </row>
     <row r="72" spans="1:25" x14ac:dyDescent="0.25">
@@ -6695,13 +6715,13 @@
         <v>3</v>
       </c>
       <c r="E72" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="F72" t="s">
-        <v>81</v>
+        <v>111</v>
       </c>
       <c r="G72" t="s">
-        <v>82</v>
+        <v>112</v>
       </c>
       <c r="H72" t="s">
         <v>189</v>
@@ -6713,25 +6733,25 @@
         <v>9</v>
       </c>
       <c r="K72" s="2">
-        <v>60080164</v>
+        <v>15037055</v>
       </c>
       <c r="L72" s="2">
-        <v>0</v>
+        <v>10235715</v>
       </c>
       <c r="M72" s="2">
-        <v>0</v>
+        <v>8519043</v>
       </c>
       <c r="N72" s="2">
         <v>0</v>
       </c>
       <c r="O72" s="2">
-        <v>0</v>
+        <v>29470499</v>
       </c>
       <c r="P72" s="2">
         <v>0</v>
       </c>
       <c r="Q72" s="2">
-        <v>60080164</v>
+        <v>63262312</v>
       </c>
       <c r="R72" s="2">
         <v>0</v>
@@ -6766,19 +6786,19 @@
         <v>1</v>
       </c>
       <c r="C73" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D73" t="s">
         <v>3</v>
       </c>
       <c r="E73" t="s">
-        <v>4</v>
+        <v>110</v>
       </c>
       <c r="F73" t="s">
-        <v>15</v>
+        <v>81</v>
       </c>
       <c r="G73" t="s">
-        <v>16</v>
+        <v>82</v>
       </c>
       <c r="H73" t="s">
         <v>191</v>
@@ -6790,7 +6810,7 @@
         <v>9</v>
       </c>
       <c r="K73" s="2">
-        <v>24122016</v>
+        <v>60080164</v>
       </c>
       <c r="L73" s="2">
         <v>0</v>
@@ -6808,7 +6828,7 @@
         <v>0</v>
       </c>
       <c r="Q73" s="2">
-        <v>24122016</v>
+        <v>60080164</v>
       </c>
       <c r="R73" s="2">
         <v>0</v>
@@ -6843,19 +6863,19 @@
         <v>1</v>
       </c>
       <c r="C74" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D74" t="s">
         <v>3</v>
       </c>
       <c r="E74" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F74" t="s">
-        <v>126</v>
+        <v>15</v>
       </c>
       <c r="G74" t="s">
-        <v>127</v>
+        <v>16</v>
       </c>
       <c r="H74" t="s">
         <v>193</v>
@@ -6867,7 +6887,7 @@
         <v>9</v>
       </c>
       <c r="K74" s="2">
-        <v>47527794</v>
+        <v>24122016</v>
       </c>
       <c r="L74" s="2">
         <v>0</v>
@@ -6885,7 +6905,7 @@
         <v>0</v>
       </c>
       <c r="Q74" s="2">
-        <v>47527794</v>
+        <v>24122016</v>
       </c>
       <c r="R74" s="2">
         <v>0</v>
@@ -6926,13 +6946,13 @@
         <v>3</v>
       </c>
       <c r="E75" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="F75" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="G75" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="H75" t="s">
         <v>195</v>
@@ -6944,7 +6964,7 @@
         <v>9</v>
       </c>
       <c r="K75" s="2">
-        <v>19090076</v>
+        <v>47527794</v>
       </c>
       <c r="L75" s="2">
         <v>0</v>
@@ -6962,7 +6982,7 @@
         <v>0</v>
       </c>
       <c r="Q75" s="2">
-        <v>19090076</v>
+        <v>47527794</v>
       </c>
       <c r="R75" s="2">
         <v>0</v>
@@ -6997,19 +7017,19 @@
         <v>1</v>
       </c>
       <c r="C76" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D76" t="s">
         <v>3</v>
       </c>
       <c r="E76" t="s">
-        <v>4</v>
+        <v>123</v>
       </c>
       <c r="F76" t="s">
-        <v>43</v>
+        <v>130</v>
       </c>
       <c r="G76" t="s">
-        <v>44</v>
+        <v>131</v>
       </c>
       <c r="H76" t="s">
         <v>197</v>
@@ -7021,7 +7041,7 @@
         <v>9</v>
       </c>
       <c r="K76" s="2">
-        <v>768791770</v>
+        <v>19090076</v>
       </c>
       <c r="L76" s="2">
         <v>0</v>
@@ -7039,7 +7059,7 @@
         <v>0</v>
       </c>
       <c r="Q76" s="2">
-        <v>768791770</v>
+        <v>19090076</v>
       </c>
       <c r="R76" s="2">
         <v>0</v>
@@ -7074,19 +7094,19 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D77" t="s">
         <v>3</v>
       </c>
       <c r="E77" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F77" t="s">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="G77" t="s">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="H77" t="s">
         <v>199</v>
@@ -7098,7 +7118,7 @@
         <v>9</v>
       </c>
       <c r="K77" s="2">
-        <v>18664603</v>
+        <v>768791770</v>
       </c>
       <c r="L77" s="2">
         <v>0</v>
@@ -7107,7 +7127,7 @@
         <v>0</v>
       </c>
       <c r="N77" s="2">
-        <v>1764004</v>
+        <v>0</v>
       </c>
       <c r="O77" s="2">
         <v>0</v>
@@ -7116,7 +7136,7 @@
         <v>0</v>
       </c>
       <c r="Q77" s="2">
-        <v>20428607</v>
+        <v>768791770</v>
       </c>
       <c r="R77" s="2">
         <v>0</v>
@@ -7151,19 +7171,19 @@
         <v>1</v>
       </c>
       <c r="C78" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D78" t="s">
         <v>3</v>
       </c>
       <c r="E78" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F78" t="s">
-        <v>10</v>
+        <v>81</v>
       </c>
       <c r="G78" t="s">
-        <v>11</v>
+        <v>82</v>
       </c>
       <c r="H78" t="s">
         <v>201</v>
@@ -7175,16 +7195,16 @@
         <v>9</v>
       </c>
       <c r="K78" s="2">
-        <v>242095176</v>
+        <v>18664603</v>
       </c>
       <c r="L78" s="2">
-        <v>132300648</v>
+        <v>0</v>
       </c>
       <c r="M78" s="2">
         <v>0</v>
       </c>
       <c r="N78" s="2">
-        <v>0</v>
+        <v>1764004</v>
       </c>
       <c r="O78" s="2">
         <v>0</v>
@@ -7193,7 +7213,7 @@
         <v>0</v>
       </c>
       <c r="Q78" s="2">
-        <v>374395824</v>
+        <v>20428607</v>
       </c>
       <c r="R78" s="2">
         <v>0</v>
@@ -7202,7 +7222,7 @@
         <v>0</v>
       </c>
       <c r="T78" s="2">
-        <v>52586280</v>
+        <v>0</v>
       </c>
       <c r="U78" s="2">
         <v>0</v>
@@ -7217,7 +7237,7 @@
         <v>0</v>
       </c>
       <c r="Y78" s="2">
-        <v>52586280</v>
+        <v>0</v>
       </c>
     </row>
     <row r="79" spans="1:25" x14ac:dyDescent="0.25">
@@ -7237,10 +7257,10 @@
         <v>4</v>
       </c>
       <c r="F79" t="s">
-        <v>181</v>
+        <v>10</v>
       </c>
       <c r="G79" t="s">
-        <v>182</v>
+        <v>11</v>
       </c>
       <c r="H79" t="s">
         <v>203</v>
@@ -7252,10 +7272,10 @@
         <v>9</v>
       </c>
       <c r="K79" s="2">
-        <v>0</v>
+        <v>242095176</v>
       </c>
       <c r="L79" s="2">
-        <v>64740000</v>
+        <v>132300648</v>
       </c>
       <c r="M79" s="2">
         <v>0</v>
@@ -7270,7 +7290,7 @@
         <v>0</v>
       </c>
       <c r="Q79" s="2">
-        <v>64740000</v>
+        <v>374395824</v>
       </c>
       <c r="R79" s="2">
         <v>0</v>
@@ -7279,7 +7299,7 @@
         <v>0</v>
       </c>
       <c r="T79" s="2">
-        <v>0</v>
+        <v>52586280</v>
       </c>
       <c r="U79" s="2">
         <v>0</v>
@@ -7294,7 +7314,7 @@
         <v>0</v>
       </c>
       <c r="Y79" s="2">
-        <v>0</v>
+        <v>52586280</v>
       </c>
     </row>
     <row r="80" spans="1:25" x14ac:dyDescent="0.25">
@@ -7305,19 +7325,19 @@
         <v>1</v>
       </c>
       <c r="C80" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D80" t="s">
         <v>3</v>
       </c>
       <c r="E80" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F80" t="s">
-        <v>126</v>
+        <v>183</v>
       </c>
       <c r="G80" t="s">
-        <v>127</v>
+        <v>184</v>
       </c>
       <c r="H80" t="s">
         <v>205</v>
@@ -7332,13 +7352,13 @@
         <v>0</v>
       </c>
       <c r="L80" s="2">
-        <v>45331549</v>
+        <v>64740000</v>
       </c>
       <c r="M80" s="2">
         <v>0</v>
       </c>
       <c r="N80" s="2">
-        <v>47387128</v>
+        <v>0</v>
       </c>
       <c r="O80" s="2">
         <v>0</v>
@@ -7347,7 +7367,7 @@
         <v>0</v>
       </c>
       <c r="Q80" s="2">
-        <v>92718677</v>
+        <v>64740000</v>
       </c>
       <c r="R80" s="2">
         <v>0</v>
@@ -7391,10 +7411,10 @@
         <v>80</v>
       </c>
       <c r="F81" t="s">
-        <v>149</v>
+        <v>130</v>
       </c>
       <c r="G81" t="s">
-        <v>150</v>
+        <v>131</v>
       </c>
       <c r="H81" t="s">
         <v>207</v>
@@ -7406,16 +7426,16 @@
         <v>9</v>
       </c>
       <c r="K81" s="2">
-        <v>115727621</v>
+        <v>0</v>
       </c>
       <c r="L81" s="2">
-        <v>0</v>
+        <v>45331549</v>
       </c>
       <c r="M81" s="2">
         <v>0</v>
       </c>
       <c r="N81" s="2">
-        <v>0</v>
+        <v>47387128</v>
       </c>
       <c r="O81" s="2">
         <v>0</v>
@@ -7424,7 +7444,7 @@
         <v>0</v>
       </c>
       <c r="Q81" s="2">
-        <v>115727621</v>
+        <v>92718677</v>
       </c>
       <c r="R81" s="2">
         <v>0</v>
@@ -7459,31 +7479,31 @@
         <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D82" t="s">
         <v>3</v>
       </c>
       <c r="E82" t="s">
+        <v>80</v>
+      </c>
+      <c r="F82" t="s">
+        <v>151</v>
+      </c>
+      <c r="G82" t="s">
+        <v>152</v>
+      </c>
+      <c r="H82" t="s">
         <v>209</v>
       </c>
-      <c r="F82" t="s">
-        <v>43</v>
-      </c>
-      <c r="G82" t="s">
-        <v>44</v>
-      </c>
-      <c r="H82" t="s">
+      <c r="I82" t="s">
         <v>210</v>
       </c>
-      <c r="I82" t="s">
-        <v>211</v>
-      </c>
       <c r="J82" t="s">
         <v>9</v>
       </c>
       <c r="K82" s="2">
-        <v>151200000</v>
+        <v>115727621</v>
       </c>
       <c r="L82" s="2">
         <v>0</v>
@@ -7501,7 +7521,7 @@
         <v>0</v>
       </c>
       <c r="Q82" s="2">
-        <v>151200000</v>
+        <v>115727621</v>
       </c>
       <c r="R82" s="2">
         <v>0</v>
@@ -7536,19 +7556,19 @@
         <v>1</v>
       </c>
       <c r="C83" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D83" t="s">
         <v>3</v>
       </c>
       <c r="E83" t="s">
-        <v>85</v>
+        <v>211</v>
       </c>
       <c r="F83" t="s">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="G83" t="s">
-        <v>82</v>
+        <v>44</v>
       </c>
       <c r="H83" t="s">
         <v>212</v>
@@ -7560,10 +7580,10 @@
         <v>9</v>
       </c>
       <c r="K83" s="2">
-        <v>1533149</v>
+        <v>151200000</v>
       </c>
       <c r="L83" s="2">
-        <v>709159</v>
+        <v>0</v>
       </c>
       <c r="M83" s="2">
         <v>0</v>
@@ -7578,10 +7598,10 @@
         <v>0</v>
       </c>
       <c r="Q83" s="2">
-        <v>2242308</v>
+        <v>151200000</v>
       </c>
       <c r="R83" s="2">
-        <v>839744</v>
+        <v>0</v>
       </c>
       <c r="S83" s="2">
         <v>0</v>
@@ -7602,7 +7622,7 @@
         <v>0</v>
       </c>
       <c r="Y83" s="2">
-        <v>839744</v>
+        <v>0</v>
       </c>
     </row>
     <row r="84" spans="1:25" x14ac:dyDescent="0.25">
@@ -7619,13 +7639,13 @@
         <v>3</v>
       </c>
       <c r="E84" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="F84" t="s">
-        <v>149</v>
+        <v>81</v>
       </c>
       <c r="G84" t="s">
-        <v>150</v>
+        <v>82</v>
       </c>
       <c r="H84" t="s">
         <v>214</v>
@@ -7637,10 +7657,10 @@
         <v>9</v>
       </c>
       <c r="K84" s="2">
-        <v>-302587</v>
+        <v>1533149</v>
       </c>
       <c r="L84" s="2">
-        <v>0</v>
+        <v>709159</v>
       </c>
       <c r="M84" s="2">
         <v>0</v>
@@ -7655,10 +7675,10 @@
         <v>0</v>
       </c>
       <c r="Q84" s="2">
-        <v>-302587</v>
+        <v>2242308</v>
       </c>
       <c r="R84" s="2">
-        <v>0</v>
+        <v>839744</v>
       </c>
       <c r="S84" s="2">
         <v>0</v>
@@ -7679,7 +7699,7 @@
         <v>0</v>
       </c>
       <c r="Y84" s="2">
-        <v>0</v>
+        <v>839744</v>
       </c>
     </row>
     <row r="85" spans="1:25" x14ac:dyDescent="0.25">
@@ -7690,31 +7710,31 @@
         <v>1</v>
       </c>
       <c r="C85" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D85" t="s">
         <v>3</v>
       </c>
       <c r="E85" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F85" t="s">
+        <v>151</v>
+      </c>
+      <c r="G85" t="s">
+        <v>152</v>
+      </c>
+      <c r="H85" t="s">
         <v>216</v>
       </c>
-      <c r="G85" t="s">
-        <v>3</v>
-      </c>
-      <c r="H85" t="s">
+      <c r="I85" t="s">
         <v>217</v>
       </c>
-      <c r="I85" t="s">
-        <v>218</v>
-      </c>
       <c r="J85" t="s">
         <v>9</v>
       </c>
       <c r="K85" s="2">
-        <v>1662768</v>
+        <v>-302587</v>
       </c>
       <c r="L85" s="2">
         <v>0</v>
@@ -7732,7 +7752,7 @@
         <v>0</v>
       </c>
       <c r="Q85" s="2">
-        <v>1662768</v>
+        <v>-302587</v>
       </c>
       <c r="R85" s="2">
         <v>0</v>
@@ -7767,19 +7787,19 @@
         <v>1</v>
       </c>
       <c r="C86" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D86" t="s">
         <v>3</v>
       </c>
       <c r="E86" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F86" t="s">
-        <v>102</v>
+        <v>218</v>
       </c>
       <c r="G86" t="s">
-        <v>103</v>
+        <v>3</v>
       </c>
       <c r="H86" t="s">
         <v>219</v>
@@ -7791,10 +7811,10 @@
         <v>9</v>
       </c>
       <c r="K86" s="2">
-        <v>0</v>
+        <v>1662768</v>
       </c>
       <c r="L86" s="2">
-        <v>6514266</v>
+        <v>0</v>
       </c>
       <c r="M86" s="2">
         <v>0</v>
@@ -7809,7 +7829,7 @@
         <v>0</v>
       </c>
       <c r="Q86" s="2">
-        <v>6514266</v>
+        <v>1662768</v>
       </c>
       <c r="R86" s="2">
         <v>0</v>
@@ -7844,19 +7864,19 @@
         <v>1</v>
       </c>
       <c r="C87" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D87" t="s">
         <v>3</v>
       </c>
       <c r="E87" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F87" t="s">
-        <v>15</v>
+        <v>106</v>
       </c>
       <c r="G87" t="s">
-        <v>16</v>
+        <v>107</v>
       </c>
       <c r="H87" t="s">
         <v>221</v>
@@ -7868,10 +7888,10 @@
         <v>9</v>
       </c>
       <c r="K87" s="2">
-        <v>11337408</v>
+        <v>0</v>
       </c>
       <c r="L87" s="2">
-        <v>0</v>
+        <v>6514266</v>
       </c>
       <c r="M87" s="2">
         <v>0</v>
@@ -7886,7 +7906,7 @@
         <v>0</v>
       </c>
       <c r="Q87" s="2">
-        <v>11337408</v>
+        <v>6514266</v>
       </c>
       <c r="R87" s="2">
         <v>0</v>
@@ -7921,19 +7941,19 @@
         <v>1</v>
       </c>
       <c r="C88" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D88" t="s">
         <v>3</v>
       </c>
       <c r="E88" t="s">
-        <v>80</v>
+        <v>4</v>
       </c>
       <c r="F88" t="s">
-        <v>111</v>
+        <v>15</v>
       </c>
       <c r="G88" t="s">
-        <v>112</v>
+        <v>16</v>
       </c>
       <c r="H88" t="s">
         <v>223</v>
@@ -7945,7 +7965,7 @@
         <v>9</v>
       </c>
       <c r="K88" s="2">
-        <v>30879072</v>
+        <v>11337408</v>
       </c>
       <c r="L88" s="2">
         <v>0</v>
@@ -7963,7 +7983,7 @@
         <v>0</v>
       </c>
       <c r="Q88" s="2">
-        <v>30879072</v>
+        <v>11337408</v>
       </c>
       <c r="R88" s="2">
         <v>0</v>
@@ -8004,13 +8024,13 @@
         <v>3</v>
       </c>
       <c r="E89" t="s">
-        <v>119</v>
+        <v>80</v>
       </c>
       <c r="F89" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
       <c r="G89" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="H89" t="s">
         <v>225</v>
@@ -8022,10 +8042,10 @@
         <v>9</v>
       </c>
       <c r="K89" s="2">
-        <v>-1763395</v>
+        <v>30879072</v>
       </c>
       <c r="L89" s="2">
-        <v>-419266</v>
+        <v>0</v>
       </c>
       <c r="M89" s="2">
         <v>0</v>
@@ -8040,7 +8060,7 @@
         <v>0</v>
       </c>
       <c r="Q89" s="2">
-        <v>-2182661</v>
+        <v>30879072</v>
       </c>
       <c r="R89" s="2">
         <v>0</v>
@@ -8075,31 +8095,31 @@
         <v>1</v>
       </c>
       <c r="C90" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D90" t="s">
         <v>3</v>
       </c>
       <c r="E90" t="s">
+        <v>123</v>
+      </c>
+      <c r="F90" t="s">
+        <v>106</v>
+      </c>
+      <c r="G90" t="s">
+        <v>107</v>
+      </c>
+      <c r="H90" t="s">
         <v>227</v>
       </c>
-      <c r="F90" t="s">
-        <v>88</v>
-      </c>
-      <c r="G90" t="s">
-        <v>89</v>
-      </c>
-      <c r="H90" t="s">
+      <c r="I90" t="s">
         <v>228</v>
       </c>
-      <c r="I90" t="s">
-        <v>229</v>
-      </c>
       <c r="J90" t="s">
         <v>9</v>
       </c>
       <c r="K90" s="2">
-        <v>888890456</v>
+        <v>0</v>
       </c>
       <c r="L90" s="2">
         <v>0</v>
@@ -8117,10 +8137,10 @@
         <v>0</v>
       </c>
       <c r="Q90" s="2">
-        <v>888890456</v>
+        <v>0</v>
       </c>
       <c r="R90" s="2">
-        <v>0</v>
+        <v>79829676</v>
       </c>
       <c r="S90" s="2">
         <v>0</v>
@@ -8141,7 +8161,7 @@
         <v>0</v>
       </c>
       <c r="Y90" s="2">
-        <v>0</v>
+        <v>79829676</v>
       </c>
     </row>
     <row r="91" spans="1:25" x14ac:dyDescent="0.25">
@@ -8158,7 +8178,7 @@
         <v>3</v>
       </c>
       <c r="E91" t="s">
-        <v>119</v>
+        <v>85</v>
       </c>
       <c r="F91" t="s">
         <v>81</v>
@@ -8167,22 +8187,22 @@
         <v>82</v>
       </c>
       <c r="H91" t="s">
+        <v>229</v>
+      </c>
+      <c r="I91" t="s">
         <v>230</v>
       </c>
-      <c r="I91" t="s">
-        <v>231</v>
-      </c>
       <c r="J91" t="s">
         <v>9</v>
       </c>
       <c r="K91" s="2">
-        <v>-2099343</v>
+        <v>0</v>
       </c>
       <c r="L91" s="2">
         <v>0</v>
       </c>
       <c r="M91" s="2">
-        <v>-840131</v>
+        <v>0</v>
       </c>
       <c r="N91" s="2">
         <v>0</v>
@@ -8194,10 +8214,10 @@
         <v>0</v>
       </c>
       <c r="Q91" s="2">
-        <v>-2939474</v>
+        <v>0</v>
       </c>
       <c r="R91" s="2">
-        <v>0</v>
+        <v>1205763</v>
       </c>
       <c r="S91" s="2">
         <v>0</v>
@@ -8218,7 +8238,7 @@
         <v>0</v>
       </c>
       <c r="Y91" s="2">
-        <v>0</v>
+        <v>1205763</v>
       </c>
     </row>
     <row r="92" spans="1:25" x14ac:dyDescent="0.25">
@@ -8229,19 +8249,19 @@
         <v>1</v>
       </c>
       <c r="C92" t="s">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="D92" t="s">
         <v>3</v>
       </c>
       <c r="E92" t="s">
-        <v>106</v>
+        <v>231</v>
       </c>
       <c r="F92" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="G92" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="H92" t="s">
         <v>232</v>
@@ -8253,10 +8273,10 @@
         <v>9</v>
       </c>
       <c r="K92" s="2">
-        <v>0</v>
+        <v>888890456</v>
       </c>
       <c r="L92" s="2">
-        <v>-913478</v>
+        <v>0</v>
       </c>
       <c r="M92" s="2">
         <v>0</v>
@@ -8265,13 +8285,13 @@
         <v>0</v>
       </c>
       <c r="O92" s="2">
-        <v>-1010177</v>
+        <v>0</v>
       </c>
       <c r="P92" s="2">
-        <v>-40971</v>
+        <v>0</v>
       </c>
       <c r="Q92" s="2">
-        <v>-1964626</v>
+        <v>888890456</v>
       </c>
       <c r="R92" s="2">
         <v>0</v>
@@ -8312,7 +8332,7 @@
         <v>3</v>
       </c>
       <c r="E93" t="s">
-        <v>80</v>
+        <v>123</v>
       </c>
       <c r="F93" t="s">
         <v>81</v>
@@ -8330,13 +8350,13 @@
         <v>9</v>
       </c>
       <c r="K93" s="2">
-        <v>0</v>
+        <v>-2099343</v>
       </c>
       <c r="L93" s="2">
         <v>0</v>
       </c>
       <c r="M93" s="2">
-        <v>0</v>
+        <v>-840131</v>
       </c>
       <c r="N93" s="2">
         <v>0</v>
@@ -8345,10 +8365,10 @@
         <v>0</v>
       </c>
       <c r="P93" s="2">
-        <v>-403920</v>
+        <v>0</v>
       </c>
       <c r="Q93" s="2">
-        <v>-403920</v>
+        <v>-2939474</v>
       </c>
       <c r="R93" s="2">
         <v>0</v>
@@ -8383,19 +8403,19 @@
         <v>1</v>
       </c>
       <c r="C94" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D94" t="s">
         <v>3</v>
       </c>
       <c r="E94" t="s">
-        <v>4</v>
+        <v>110</v>
       </c>
       <c r="F94" t="s">
-        <v>5</v>
+        <v>81</v>
       </c>
       <c r="G94" t="s">
-        <v>6</v>
+        <v>82</v>
       </c>
       <c r="H94" t="s">
         <v>236</v>
@@ -8407,10 +8427,10 @@
         <v>9</v>
       </c>
       <c r="K94" s="2">
-        <v>10069920</v>
+        <v>0</v>
       </c>
       <c r="L94" s="2">
-        <v>0</v>
+        <v>-913478</v>
       </c>
       <c r="M94" s="2">
         <v>0</v>
@@ -8419,19 +8439,19 @@
         <v>0</v>
       </c>
       <c r="O94" s="2">
-        <v>0</v>
+        <v>-1010177</v>
       </c>
       <c r="P94" s="2">
-        <v>0</v>
+        <v>-40971</v>
       </c>
       <c r="Q94" s="2">
-        <v>10069920</v>
+        <v>-1964626</v>
       </c>
       <c r="R94" s="2">
         <v>0</v>
       </c>
       <c r="S94" s="2">
-        <v>10069920</v>
+        <v>0</v>
       </c>
       <c r="T94" s="2">
         <v>0</v>
@@ -8449,7 +8469,7 @@
         <v>0</v>
       </c>
       <c r="Y94" s="2">
-        <v>10069920</v>
+        <v>0</v>
       </c>
     </row>
     <row r="95" spans="1:25" x14ac:dyDescent="0.25">
@@ -8460,19 +8480,19 @@
         <v>1</v>
       </c>
       <c r="C95" t="s">
-        <v>2</v>
+        <v>79</v>
       </c>
       <c r="D95" t="s">
         <v>3</v>
       </c>
       <c r="E95" t="s">
-        <v>4</v>
+        <v>80</v>
       </c>
       <c r="F95" t="s">
-        <v>43</v>
+        <v>81</v>
       </c>
       <c r="G95" t="s">
-        <v>44</v>
+        <v>82</v>
       </c>
       <c r="H95" t="s">
         <v>238</v>
@@ -8484,7 +8504,7 @@
         <v>9</v>
       </c>
       <c r="K95" s="2">
-        <v>4448736</v>
+        <v>0</v>
       </c>
       <c r="L95" s="2">
         <v>0</v>
@@ -8499,16 +8519,16 @@
         <v>0</v>
       </c>
       <c r="P95" s="2">
-        <v>0</v>
+        <v>-403920</v>
       </c>
       <c r="Q95" s="2">
-        <v>4448736</v>
+        <v>-403920</v>
       </c>
       <c r="R95" s="2">
         <v>0</v>
       </c>
       <c r="S95" s="2">
-        <v>4448736</v>
+        <v>0</v>
       </c>
       <c r="T95" s="2">
         <v>0</v>
@@ -8526,7 +8546,7 @@
         <v>0</v>
       </c>
       <c r="Y95" s="2">
-        <v>4448736</v>
+        <v>0</v>
       </c>
     </row>
     <row r="96" spans="1:25" x14ac:dyDescent="0.25">
@@ -8561,7 +8581,7 @@
         <v>9</v>
       </c>
       <c r="K96" s="2">
-        <v>37748160</v>
+        <v>10069920</v>
       </c>
       <c r="L96" s="2">
         <v>0</v>
@@ -8579,13 +8599,13 @@
         <v>0</v>
       </c>
       <c r="Q96" s="2">
-        <v>37748160</v>
+        <v>10069920</v>
       </c>
       <c r="R96" s="2">
         <v>0</v>
       </c>
       <c r="S96" s="2">
-        <v>37748160</v>
+        <v>10069920</v>
       </c>
       <c r="T96" s="2">
         <v>0</v>
@@ -8603,7 +8623,7 @@
         <v>0</v>
       </c>
       <c r="Y96" s="2">
-        <v>37748160</v>
+        <v>10069920</v>
       </c>
     </row>
     <row r="97" spans="1:25" x14ac:dyDescent="0.25">
@@ -8623,10 +8643,10 @@
         <v>4</v>
       </c>
       <c r="F97" t="s">
-        <v>49</v>
+        <v>43</v>
       </c>
       <c r="G97" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="H97" t="s">
         <v>242</v>
@@ -8638,7 +8658,7 @@
         <v>9</v>
       </c>
       <c r="K97" s="2">
-        <v>11043605</v>
+        <v>4448736</v>
       </c>
       <c r="L97" s="2">
         <v>0</v>
@@ -8656,13 +8676,13 @@
         <v>0</v>
       </c>
       <c r="Q97" s="2">
-        <v>11043605</v>
+        <v>4448736</v>
       </c>
       <c r="R97" s="2">
         <v>0</v>
       </c>
       <c r="S97" s="2">
-        <v>11043605</v>
+        <v>4448736</v>
       </c>
       <c r="T97" s="2">
         <v>0</v>
@@ -8680,7 +8700,7 @@
         <v>0</v>
       </c>
       <c r="Y97" s="2">
-        <v>11043605</v>
+        <v>4448736</v>
       </c>
     </row>
     <row r="98" spans="1:25" x14ac:dyDescent="0.25">
@@ -8854,7 +8874,7 @@
         <v>80</v>
       </c>
       <c r="F100" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="G100" t="s">
         <v>3</v>
@@ -8914,8 +8934,239 @@
         <v>600480</v>
       </c>
     </row>
+    <row r="101" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>0</v>
+      </c>
+      <c r="B101" t="s">
+        <v>1</v>
+      </c>
+      <c r="C101" t="s">
+        <v>2</v>
+      </c>
+      <c r="D101" t="s">
+        <v>3</v>
+      </c>
+      <c r="E101" t="s">
+        <v>4</v>
+      </c>
+      <c r="F101" t="s">
+        <v>49</v>
+      </c>
+      <c r="G101" t="s">
+        <v>50</v>
+      </c>
+      <c r="H101" t="s">
+        <v>248</v>
+      </c>
+      <c r="I101" t="s">
+        <v>249</v>
+      </c>
+      <c r="J101" t="s">
+        <v>9</v>
+      </c>
+      <c r="K101" s="2">
+        <v>15683328</v>
+      </c>
+      <c r="L101" s="2">
+        <v>0</v>
+      </c>
+      <c r="M101" s="2">
+        <v>0</v>
+      </c>
+      <c r="N101" s="2">
+        <v>0</v>
+      </c>
+      <c r="O101" s="2">
+        <v>0</v>
+      </c>
+      <c r="P101" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q101" s="2">
+        <v>15683328</v>
+      </c>
+      <c r="R101" s="2">
+        <v>0</v>
+      </c>
+      <c r="S101" s="2">
+        <v>15683328</v>
+      </c>
+      <c r="T101" s="2">
+        <v>0</v>
+      </c>
+      <c r="U101" s="2">
+        <v>0</v>
+      </c>
+      <c r="V101" s="2">
+        <v>0</v>
+      </c>
+      <c r="W101" s="2">
+        <v>0</v>
+      </c>
+      <c r="X101" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y101" s="2">
+        <v>15683328</v>
+      </c>
+    </row>
+    <row r="102" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
+        <v>0</v>
+      </c>
+      <c r="B102" t="s">
+        <v>1</v>
+      </c>
+      <c r="C102" t="s">
+        <v>2</v>
+      </c>
+      <c r="D102" t="s">
+        <v>3</v>
+      </c>
+      <c r="E102" t="s">
+        <v>4</v>
+      </c>
+      <c r="F102" t="s">
+        <v>43</v>
+      </c>
+      <c r="G102" t="s">
+        <v>44</v>
+      </c>
+      <c r="H102" t="s">
+        <v>250</v>
+      </c>
+      <c r="I102" t="s">
+        <v>251</v>
+      </c>
+      <c r="J102" t="s">
+        <v>9</v>
+      </c>
+      <c r="K102" s="2">
+        <v>5766638</v>
+      </c>
+      <c r="L102" s="2">
+        <v>0</v>
+      </c>
+      <c r="M102" s="2">
+        <v>0</v>
+      </c>
+      <c r="N102" s="2">
+        <v>0</v>
+      </c>
+      <c r="O102" s="2">
+        <v>0</v>
+      </c>
+      <c r="P102" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q102" s="2">
+        <v>5766638</v>
+      </c>
+      <c r="R102" s="2">
+        <v>0</v>
+      </c>
+      <c r="S102" s="2">
+        <v>5766638</v>
+      </c>
+      <c r="T102" s="2">
+        <v>0</v>
+      </c>
+      <c r="U102" s="2">
+        <v>0</v>
+      </c>
+      <c r="V102" s="2">
+        <v>0</v>
+      </c>
+      <c r="W102" s="2">
+        <v>0</v>
+      </c>
+      <c r="X102" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y102" s="2">
+        <v>5766638</v>
+      </c>
+    </row>
+    <row r="103" spans="1:25" x14ac:dyDescent="0.25">
+      <c r="A103" t="s">
+        <v>0</v>
+      </c>
+      <c r="B103" t="s">
+        <v>1</v>
+      </c>
+      <c r="C103" t="s">
+        <v>2</v>
+      </c>
+      <c r="D103" t="s">
+        <v>3</v>
+      </c>
+      <c r="E103" t="s">
+        <v>231</v>
+      </c>
+      <c r="F103" t="s">
+        <v>10</v>
+      </c>
+      <c r="G103" t="s">
+        <v>11</v>
+      </c>
+      <c r="H103" t="s">
+        <v>252</v>
+      </c>
+      <c r="I103" t="s">
+        <v>253</v>
+      </c>
+      <c r="J103" t="s">
+        <v>9</v>
+      </c>
+      <c r="K103" s="2">
+        <v>0</v>
+      </c>
+      <c r="L103" s="2">
+        <v>0</v>
+      </c>
+      <c r="M103" s="2">
+        <v>0</v>
+      </c>
+      <c r="N103" s="2">
+        <v>0</v>
+      </c>
+      <c r="O103" s="2">
+        <v>0</v>
+      </c>
+      <c r="P103" s="2">
+        <v>0</v>
+      </c>
+      <c r="Q103" s="2">
+        <v>0</v>
+      </c>
+      <c r="R103" s="2">
+        <v>2002946</v>
+      </c>
+      <c r="S103" s="2">
+        <v>0</v>
+      </c>
+      <c r="T103" s="2">
+        <v>0</v>
+      </c>
+      <c r="U103" s="2">
+        <v>0</v>
+      </c>
+      <c r="V103" s="2">
+        <v>0</v>
+      </c>
+      <c r="W103" s="2">
+        <v>0</v>
+      </c>
+      <c r="X103" s="2">
+        <v>0</v>
+      </c>
+      <c r="Y103" s="2">
+        <v>2002946</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Y100"/>
+  <autoFilter ref="A1:Y103"/>
   <phoneticPr fontId="0" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter alignWithMargins="0"/>

</xml_diff>